<commit_message>
arch and req without fixes
</commit_message>
<xml_diff>
--- a/outputs/evaluation/architecture/CF_M01_arch_eval.xlsx
+++ b/outputs/evaluation/architecture/CF_M01_arch_eval.xlsx
@@ -447,14 +447,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>all elements (name | isPartOf)</t>
+          <t>all elements (units/patterns by name, connectors by unit-pair)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.7609</v>
+        <v>0.7045</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7609</v>
+        <v>0.7949000000000001</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -469,13 +469,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.7188</v>
+        <v>0.9286</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7931</v>
+        <v>0.7879</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8998</v>
+        <v>0.9714</v>
       </c>
     </row>
     <row r="6">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.9429</v>
+        <v>0.931</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -517,10 +517,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.6857</v>
+        <v>0.7931</v>
       </c>
       <c r="C8" t="n">
-        <v>0.5511</v>
+        <v>0.8115</v>
       </c>
     </row>
     <row r="9">
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.8286</v>
+        <v>0.8276</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.9667</v>
+        <v>0.5385</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -559,10 +559,8 @@
           <t>fixes</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B11" t="n">
+        <v>0</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -623,19 +621,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C2" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D2" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7407</v>
+        <v>0.92</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7407</v>
+        <v>0.8214</v>
       </c>
     </row>
     <row r="3">
@@ -648,13 +646,13 @@
         <v>4</v>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
         <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
         <v>0.75</v>
@@ -663,23 +661,23 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>connector (unit-pairs)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="C4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D4" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>0.8571</v>
+        <v>0.3125</v>
       </c>
       <c r="F4" t="n">
-        <v>0.8</v>
+        <v>0.7143</v>
       </c>
     </row>
   </sheetData>
@@ -693,7 +691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -715,7 +713,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
@@ -725,77 +723,101 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>True Positives (matched)</t>
+          <t>True Positives (matched elements)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Validated correct (name for units/patterns, isPartOf for connectors)</t>
+          <t>Named correct (units/patterns by name)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>35</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>False Positives</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>11</v>
+          <t>Connector unit-pairs (GT / LLM)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>7 / 16</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>False Negatives</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>11</v>
+          <t>Connector pair TP (recall / precision)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>5 / 5</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Precision (all elements; units/patterns by name, connectors by isPartOf)</t>
+          <t>False Positives</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.7609</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Recall (all elements; units/patterns by name, connectors by isPartOf)</t>
+          <t>False Negatives</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.7609</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Precision (units/patterns by name, connectors by unit-pair)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.7045</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Recall (units/patterns by name, connectors by unit-pair)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.7949000000000001</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Match threshold (cosine)</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>0.35</v>
+      <c r="B12" t="n">
+        <v>0.75</v>
       </c>
     </row>
   </sheetData>
@@ -861,25 +883,25 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>33</v>
+      </c>
+      <c r="C2" t="n">
+        <v>28</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26</v>
+      </c>
+      <c r="E2" t="n">
+        <v>26</v>
+      </c>
+      <c r="F2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G2" t="n">
+        <v>26</v>
+      </c>
+      <c r="H2" t="n">
         <v>29</v>
-      </c>
-      <c r="C2" t="n">
-        <v>32</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23</v>
-      </c>
-      <c r="E2" t="n">
-        <v>23</v>
-      </c>
-      <c r="F2" t="n">
-        <v>23</v>
-      </c>
-      <c r="G2" t="n">
-        <v>23</v>
-      </c>
-      <c r="H2" t="n">
-        <v>35</v>
       </c>
     </row>
     <row r="3">
@@ -889,25 +911,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C3" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="D3" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E3" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F3" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G3" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="H3" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -917,25 +939,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C4" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="D4" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E4" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F4" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G4" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H4" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
@@ -945,25 +967,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C5" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="D5" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E5" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F5" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G5" t="n">
+        <v>24</v>
+      </c>
+      <c r="H5" t="n">
         <v>29</v>
-      </c>
-      <c r="H5" t="n">
-        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -973,25 +995,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C6" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D6" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E6" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F6" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G6" t="n">
+        <v>14</v>
+      </c>
+      <c r="H6" t="n">
         <v>29</v>
-      </c>
-      <c r="H6" t="n">
-        <v>35</v>
       </c>
     </row>
     <row r="7">
@@ -1004,13 +1026,13 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -1019,7 +1041,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1033,7 +1055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T36"/>
+  <dimension ref="A1:T30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1141,12 +1163,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AU_04</t>
+          <t>AU_19</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CF_M01_AU08</t>
+          <t>CF_M01_AU01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1155,67 +1177,63 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.6546</v>
+        <v>0.7799</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Web Platform</t>
+          <t>User</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Web interface for the Waapiti platform.</t>
+          <t>El client és l’usuari de la plataforma.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>['AU_01']</t>
-        </is>
-      </c>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>AU_04</t>
+          <t>AU_19</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Web platform interface</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>In the case of this layer, you can see that it is made up of the interface of the web platform and the Waapiti mobile platform.</t>
+          <t>The client is the user of the platform</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>CF_M01_AU05</t>
+          <t>CF_M01_P01</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>CF_M01_AU08</t>
+          <t>CF_M01_AU01</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
@@ -1223,12 +1241,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AU_07</t>
+          <t>AU_17</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CF_M01_AU11</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1237,43 +1255,43 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.6583</v>
+        <v>0.8603</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Main service responsible for the platform's core business logic.</t>
+          <t>Per la infraestructura es farà ús dels serveis cloud d’AWS.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>['AU_02']</t>
+          <t>['AU_03']</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>AU_07</t>
+          <t>AU_17</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Core Service</t>
+          <t>AWS cloud services set</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -1283,21 +1301,23 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>This service is responsible for carrying out the business logic of the platform, it would be the main core of the platform. Mainly, it interacts with the database, although it also interacts to a lesser extent with cloud services.</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
-        <v>44</v>
+          <t>As can be seen in Figure 9.1, the data layer is made up of AWS cloud services and the database. […] The objective of these services is to form a data lake where all the historical data is stored in order to process them in the analytical module.</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>44, 45</t>
+        </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_AU07</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>CF_M01_AU11</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
@@ -1310,7 +1330,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CF_M01_AU09</t>
+          <t>CF_M01_AU11</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1319,31 +1339,31 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.7151</v>
+        <v>0.8605</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Mobile Platform</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Mobile interface for the Waapiti platform.</t>
+          <t>Servei Core: Aquest servei s’encarrega de realitzar la lògica de negoci de la plataforma, seria el nucli principal de la plataforma.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>['AU_01']</t>
+          <t>['AU_02']</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -1355,7 +1375,7 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Waapiti Mobile Platform</t>
+          <t>Core Service</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -1365,21 +1385,21 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>In the case of this layer, you can see that it is made up of the interface of the web platform and the Waapiti mobile platform.</t>
+          <t>This service is responsible for carrying out the business logic of the platform, it would be the main core of the platform. Mainly, it interacts with the database, although it also interacts to a lesser extent with cloud services.</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>CF_M01_AU05</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>CF_M01_AU09</t>
+          <t>CF_M01_AU11</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
@@ -1387,12 +1407,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AU_12</t>
+          <t>AU_09</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_AU15</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1401,11 +1421,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.7651</v>
+        <v>0.8633</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Cloud Services</t>
+          <t>Database</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1415,12 +1435,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Collection of AWS services forming a data lake for historical data processing.</t>
+          <t>Base de dades: La base de dades utilitzada és una base de dades MySQL que s’encarrega d’emmagatzemar totes les dades necessàries per al funcionament del sistema.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1431,29 +1451,27 @@
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>AU_12</t>
+          <t>AU_09</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>AWS cloud services set</t>
+          <t>SQL database</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Component</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>As can be seen in Figure 9.1, the data layer is made up of AWS cloud services and the database. […] The objective of these services is to form a data lake where all the historical data is stored in order to process them in the analytical module.</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>44, 45</t>
-        </is>
+          <t>As can be seen in Figure 9.1, the data layer is made up of AWS cloud services and the database. [...] The database used is a MySQL database that is responsible for storing all the data necessary for the operation of the system. This database is implemented in the RDS service [30], which is a distributed relational database service from AWS.</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>44</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -1463,7 +1481,7 @@
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_AU15</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
@@ -1471,7 +1489,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AU_06</t>
+          <t>AU_04</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1485,7 +1503,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.7959000000000001</v>
+        <v>0.9471000000000001</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1499,23 +1517,23 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Service responsible for management, authentication, and authorization of users, acting as the entry point for the business layer.</t>
+          <t>L’únic component que interactua de manera directa amb la capa de presentació és el mòdul Api Gateway.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>43, 44</t>
+          <t>43</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>['AU_02']</t>
+          <t>['P_03']</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>AU_06</t>
+          <t>AU_04</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -1553,12 +1571,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AU_11</t>
+          <t>AU_07</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CF_M01_AU15</t>
+          <t>CF_M01_AU13</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1567,21 +1585,21 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.8082</v>
+        <v>0.9573</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Database</t>
+          <t>API Player</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Relational database storing system data.</t>
+          <t>Api Player: Aquest servei s’encarrega de comunicar-se amb els players rebent tota la informació corresponent a aquest.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1591,29 +1609,29 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>['AU_03']</t>
+          <t>['AU_02']</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>AU_11</t>
+          <t>AU_07</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>SQL database</t>
+          <t>Api Player</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>As can be seen in Figure 9.1, the data layer is made up of AWS cloud services and the database. [...] The database used is a MySQL database that is responsible for storing all the data necessary for the operation of the system. This database is implemented in the RDS service [30], which is a distributed relational database service from AWS.</t>
+          <t>This service is responsible for communicating with the players, receiving all the information corresponding to them. The information they can receive can be the status of the player, the contents it plays, the schedules in which these contents should be played, etc. This information is processed and stored</t>
         </is>
       </c>
       <c r="P7" t="n">
@@ -1621,13 +1639,13 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>CF_M01_AU07</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
-          <t>CF_M01_AU15</t>
+          <t>CF_M01_AU13</t>
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
@@ -1635,12 +1653,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AU_16</t>
+          <t>AU_06</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CF_M01_AU18</t>
+          <t>CF_M01_AU12</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1649,67 +1667,67 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.8250999999999999</v>
+        <v>0.9891</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>DynamoDB</t>
+          <t>Analytical Module</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>NoSQL database service used for real-time playlog storage.</t>
+          <t>Mòdul analític: Aquest servei és el servei que s’ha començat a desenvolupar durant el desenvolupament d’aquest TFG.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>45, 48</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>['AU_12']</t>
+          <t>['AU_02']</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>AU_16</t>
+          <t>AU_06</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Amazon DynamoDB</t>
+          <t>Analytical module</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>This service is a non-relational database from AWS. In our case, it is responsible for storing playlogs in real time.</t>
+          <t>Its main function is to obtain and process data from playlogs, connections and platform actions. This service mainly interacts with cloud services, although it also interacts to a lesser extent with the database.</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
         <is>
-          <t>CF_M01_AU18</t>
+          <t>CF_M01_AU12</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
@@ -1717,12 +1735,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P_02</t>
+          <t>P_03</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CF_M01_P02</t>
+          <t>CF_M01_P04</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1735,63 +1753,67 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Three Layers</t>
+          <t>API Gateway</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Architectural Pattern</t>
+          <t>Design Pattern</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The system is divided into three layers: presentation layer, business layer, and data layer.</t>
+          <t>Això és degut de què es segueix el patró de disseny de microserveis Api Gateway. Aquest patró de disseny permet que solament un component sigui qui interactuï entre els usuaris i els serveis que proporciona la plataforma.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>43</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>['P_01']</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
+          <t>['AU_02']</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>The document labels this as a 'patró de disseny de microserveis' (microservices design pattern). While it is a pattern used in microservices, it is classified here as a Design Pattern as per the provided definitions.</t>
+        </is>
+      </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>P_02</t>
+          <t>P_03</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Three Layers</t>
+          <t>API Gateway</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Architectural Pattern</t>
+          <t>Design Pattern</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>The client-server model uses a 3-layer architecture, where the system is divided into 3 layers.</t>
+          <t>This design pattern allows only one component to interact between users and the services provided by the platform.</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>CF_M01_P01</t>
+          <t>CF_M01_P03</t>
         </is>
       </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
-          <t>CF_M01_P02</t>
+          <t>CF_M01_P04</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
@@ -1799,17 +1821,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>P_01</t>
+          <t>AU_10</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CF_M01_P01</t>
+          <t>CF_M01_AU32</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>pattern</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1817,55 +1839,63 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Client-Server</t>
+          <t>MySQL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Architectural Pattern</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The platform is a web service where the client makes requests to a server that processes them and returns the response.</t>
+          <t>La base de dades utilitzada és una base de dades MySQL.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>41</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>['AU_09']</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>P_01</t>
+          <t>AU_10</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Client-Server</t>
+          <t>MySQL</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Architectural Pattern</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>The Waapiti platform is a web service that follows the client-server architecture. In this type of architecture, the client is the one who makes requests to a server, which processes them and returns the response to the client.</t>
+          <t>The database used is a MySQL database that is responsible for storing all the data necessary for the operation of the system.</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>41</v>
-      </c>
-      <c r="Q10" t="inlineStr"/>
+        <v>44</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>CF_M01_AU15</t>
+        </is>
+      </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
-          <t>CF_M01_P01</t>
+          <t>CF_M01_AU32</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
@@ -1873,12 +1903,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AU_23</t>
+          <t>AU_18</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CF_M01_AU30</t>
+          <t>CF_M01_AU27</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1901,7 +1931,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Hardware device (miniature computer) that connects screens to the platform to reproduce content.</t>
+          <t>Un player consisteix en un dispositiu que pot ser intern o extern, que permet a les pantalles reproduir continguts.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1913,7 +1943,7 @@
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>AU_23</t>
+          <t>AU_18</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -1939,7 +1969,7 @@
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr">
         <is>
-          <t>CF_M01_AU30</t>
+          <t>CF_M01_AU27</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
@@ -1947,12 +1977,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AU_19</t>
+          <t>AU_22</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CF_M01_AU22</t>
+          <t>CF_M01_AU20</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1965,7 +1995,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Kinesis Data Streams</t>
+          <t>Amazon Athena</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1975,12 +2005,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Streaming service for real-time data ingestion.</t>
+          <t>El servei d’Amazon Athena és un servei que permet realitzar consultes en SQL sobre dades emmagatzemades en Amazon S3.</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>49</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1991,13 +2021,13 @@
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>AU_19</t>
+          <t>AU_22</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Kinesis Data Streams</t>
+          <t>Amazon Athena</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -2007,13 +2037,11 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Data processing and ingestion service aimed especially at data streaming. In the development of this project, Kinesis Data Streams has been used to transmit playlog and audit trail data.</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>50, 51</t>
-        </is>
+          <t>Service that allows you to perform SQL queries on data stored in Amazon S3</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>49</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -2023,7 +2051,7 @@
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
-          <t>CF_M01_AU22</t>
+          <t>CF_M01_AU20</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
@@ -2031,12 +2059,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AU_17</t>
+          <t>AU_01</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CF_M01_AU20</t>
+          <t>CF_M01_AU05</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2049,63 +2077,63 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Amazon Athena</t>
+          <t>Presentation Layer</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Layer</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Query service for analyzing data in S3.</t>
+          <t>Capa de presentació: És la capa que s’encarrega de mostrar la informació a l’usuari.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>['AU_12']</t>
+          <t>['P_02']</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>AU_17</t>
+          <t>AU_01</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Amazon Athena</t>
+          <t>Presentation Layer</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Layer</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Service that allows you to perform SQL queries on data stored in Amazon S3</t>
+          <t>It is the layer that is responsible for displaying information to the user. In this project, it is the visual interface of the Waapiti platform.</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_P02</t>
         </is>
       </c>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
-          <t>CF_M01_AU20</t>
+          <t>CF_M01_AU05</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
@@ -2113,12 +2141,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AU_15</t>
+          <t>AU_20</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CF_M01_AU17</t>
+          <t>CF_M01_AU03</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2131,7 +2159,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Amazon S3</t>
+          <t>HTTP</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -2141,29 +2169,29 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Object storage service used for the data lake.</t>
+          <t>La comunicació entre els dos components es realitza a través d’internet mitjançant el protocol HTTP.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>45, 48</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>['AU_12']</t>
+          <t>['AU_04']</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>AU_15</t>
+          <t>AU_20</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Amazon S3</t>
+          <t>HTTP</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -2173,21 +2201,21 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>This is the AWS object storage service. In this project it is responsible for storing JSON documents containing playlogs, connections and audit trails.</t>
+          <t>Communication between the two components is carried out over the internet using the HTTP protocol and the REST API model.</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_AU24, CF_M01_AU25</t>
         </is>
       </c>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
-          <t>CF_M01_AU17</t>
+          <t>CF_M01_AU03</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
@@ -2195,172 +2223,176 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AU_10</t>
+          <t>AU_26</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CF_M01_AU14</t>
+          <t>CF_M01_AU25</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="D15" t="n">
         <v>1</v>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Web Socket</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Connector</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Service responsible for bidirectional communication between the platform and players.</t>
+          <t>L’únic component que interactua de manera directa amb la capa de presentació és el mòdul Api Gateway.</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>42,43</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>['AU_02']</t>
+          <t>['AU_04', 'AU_01']</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>AU_10</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>Web Socket</t>
-        </is>
-      </c>
+          <t>AU_26</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>api gateway, presentation layer</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Connector</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>This service is responsible for communicating between the platform and the players, thus allowing the exchange of information between them. It processes the data coming from the players and stores it in the database and in the cloud services.</t>
+          <t>more specifically with the Api Gateway</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_AU05, CF_M01_AU10</t>
         </is>
       </c>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
-          <t>CF_M01_AU14</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr"/>
+          <t>CF_M01_AU25</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>presentation layer, api gateway service</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AU_02</t>
+          <t>AU_28</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_AU26</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="D16" t="n">
         <v>1</v>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Business Layer</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Layer</t>
+          <t>Connector</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Core layer responsible for processing information and business logic.</t>
+          <t>El servei Api Gateway [...] processa les peticions per poder enviar-les al servei Core i al mòdul analític.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>41, 42</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>['AU_04', 'AU_05', 'AU_06']</t>
+        </is>
+      </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>AU_02</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Business Layer</t>
-        </is>
-      </c>
+          <t>AU_28</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>api gateway, core, analytical module</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Layer</t>
+          <t>Connector</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>This layer is the core of the application, which is responsible for processing all the information. In our context, it is the software that is responsible for processing user requests.</t>
+          <t>Furthermore, it can be observed that three components are directly or indirectly related to the presentation layer, that is, they interact with users. These components would be, the Api Gateway, the Core and the analytical module. […] the only component that interacts directly with the presentation layer is the Api Gateway module [...]</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>CF_M01_P02</t>
+          <t>CF_M01_AU10, CF_M01_AU11, CF_M01_AU12</t>
         </is>
       </c>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr"/>
+          <t>CF_M01_AU26</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>api gateway service, core service, analytical module</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AU_28</t>
+          <t>AU_31</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CF_M01_AU35</t>
+          <t>CF_M01_AU28</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2379,28 +2411,28 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>The Web Platform communicates with the API Gateway.</t>
+          <t>Api Player: Aquest servei s’encarrega de comunicar-se amb els players rebent tota la informació corresponent a aquest.</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>['AU_04', 'AU_06']</t>
+          <t>['AU_07', 'AU_18']</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>AU_28</t>
+          <t>AU_31</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>web platform, api gateway</t>
+          <t>api player, player</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
@@ -2411,877 +2443,875 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>The Web Platform communicates with the API Gateway.</t>
+          <t>This service is responsible for communicating with players.</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>CF_M01_AU10, CF_M01_AU08</t>
+          <t>CF_M01_AU27, CF_M01_AU13</t>
         </is>
       </c>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr">
         <is>
-          <t>CF_M01_AU35</t>
+          <t>CF_M01_AU28</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>api gateway service, web platform interface</t>
+          <t>player, api player</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AU_29</t>
+          <t>AU_15</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CF_M01_AU36</t>
+          <t>CF_M01_AU33</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D18" t="n">
         <v>1</v>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>NestJS</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>The Mobile Platform communicates with the API Gateway.</t>
+          <t>Com a framework es farà ús de NestJS.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>['AU_05', 'AU_06']</t>
+          <t>['AU_05']</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>AU_29</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>mobile platform, api gateway</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr"/>
+          <t>AU_15</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>NestJS</t>
+        </is>
+      </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>The Mobile Platform communicates with the API Gateway.</t>
+          <t>This framework is a NodeJS framework whose main function is to create backend applications. In this project, this framework has been used to develop the different services that interact with each other.</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>CF_M01_AU10, CF_M01_AU09</t>
+          <t>CF_M01_AU02</t>
         </is>
       </c>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
-          <t>CF_M01_AU36</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>api gateway service, waapiti mobile platform</t>
-        </is>
-      </c>
+          <t>CF_M01_AU33</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AU_30</t>
+          <t>AU_08</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CF_M01_AU26</t>
+          <t>CF_M01_AU14</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D19" t="n">
         <v>1</v>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Web Socket</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>The API Gateway communicates with the Core service.</t>
+          <t>Web Socket: Aquest servei s’encarrega de realitzar la comunicació entre la plataforma i els players, i d’aquesta manera permet l’intercanvi d’informació entre ells.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>43, 44</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>['AU_06', 'AU_07']</t>
+          <t>['AU_02']</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>AU_30</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>api gateway, core</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr"/>
+          <t>AU_08</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Web Socket</t>
+        </is>
+      </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Furthermore, it can be observed that three components are directly or indirectly related to the presentation layer, that is, they interact with users. These components would be, the Api Gateway, the Core and the analytical module. […] the only component that interacts directly with the presentation layer is the Api Gateway module [...]</t>
+          <t>This service is responsible for communicating between the platform and the players, thus allowing the exchange of information between them. It processes the data coming from the players and stores it in the database and in the cloud services.</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>CF_M01_AU10, CF_M01_AU11</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr">
         <is>
-          <t>CF_M01_AU26</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>api gateway service, core service</t>
-        </is>
-      </c>
+          <t>CF_M01_AU14</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AU_31</t>
+          <t>AU_13</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CF_M01_AU27</t>
+          <t>CF_M01_AU17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D20" t="n">
         <v>1</v>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Amazon S3</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>The API Gateway communicates with the Analytical Module.</t>
+          <t>Amazon S3: Aquest és el servei d’emmagatzament d’objectes d’AWS.</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>43, 44</t>
+          <t>45</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>['AU_06', 'AU_08']</t>
+          <t>['AU_12']</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>AU_31</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>api gateway, analytical module</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr"/>
+          <t>AU_13</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Amazon S3</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Furthermore, it can be observed that three components are directly or indirectly related to the presentation layer, that is, they interact with users. These components would be, the Api Gateway, the Core and the analytical module. […] the only component that interacts directly with the presentation layer is the Api Gateway module [...]</t>
+          <t>This is the AWS object storage service. In this project it is responsible for storing JSON documents containing playlogs, connections and audit trails.</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>CF_M01_AU10, CF_M01_AU12</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr">
         <is>
-          <t>CF_M01_AU27</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>api gateway service, analytical module</t>
-        </is>
-      </c>
+          <t>CF_M01_AU17</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AU_32</t>
+          <t>AU_23</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CF_M01_AU31</t>
+          <t>CF_M01_AU21</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D21" t="n">
         <v>1</v>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>AWS Glue</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>The Player communicates with the API Player service.</t>
+          <t>El servei d’AWS Glue és un servei d’integració de dades sense servidor.</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>49</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>['AU_23', 'AU_09']</t>
+          <t>['AU_12']</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>AU_32</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>player, api player</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr"/>
+          <t>AU_23</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>AWS Glue</t>
+        </is>
+      </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>This service is responsible for communicating with players.</t>
+          <t>Serverless data integration service that allows us to detect, prepare, migrate and integrate data from different sources. In the case of the development of this project we have made use of the AWS Glue Data Catalog function. The use of this has been necessary to be able to store the metadata of the project data</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>CF_M01_AU30, CF_M01_AU13</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr">
         <is>
-          <t>CF_M01_AU31</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>player, api player</t>
-        </is>
-      </c>
+          <t>CF_M01_AU21</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AU_33</t>
+          <t>AU_02</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CF_M01_AU32</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D22" t="n">
         <v>1</v>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Business Layer</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Layer</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>The Player communicates with the Web Socket service.</t>
+          <t>Capa de negoci: Aquesta capa és el nucli de l’aplicació, que s’encarrega de processar tota la informació.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>['AU_23', 'AU_10']</t>
+          <t>['P_02']</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>AU_33</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>player, web socket</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr"/>
+          <t>AU_02</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Business Layer</t>
+        </is>
+      </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Layer</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>This service is responsible for communicating between the platform and the players.</t>
+          <t>This layer is the core of the application, which is responsible for processing all the information. In our context, it is the software that is responsible for processing user requests.</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>CF_M01_AU30, CF_M01_AU14</t>
+          <t>CF_M01_P02</t>
         </is>
       </c>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr">
         <is>
-          <t>CF_M01_AU32</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>player, web socket</t>
-        </is>
-      </c>
+          <t>CF_M01_AU06</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AU_34</t>
+          <t>P_02</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CF_M01_AU38</t>
+          <t>CF_M01_P02</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>pattern</t>
         </is>
       </c>
       <c r="D23" t="n">
         <v>1</v>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Three Layers</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Architectural Pattern</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>The Web Socket service communicates with the Database.</t>
+          <t>Pel model client-servidor s’utilitza l’arquitectura de 3 capes, on el sistema es devidiex en 3 capes, la capa de presentació, la capa de negoci i la capa de dades.</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>['AU_10', 'AU_11']</t>
+          <t>['P_01']</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>AU_34</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>web socket, database</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr"/>
+          <t>P_02</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Three Layers</t>
+        </is>
+      </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Architectural Pattern</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>The Web Socket service communicates with the Database.</t>
+          <t>The client-server model uses a 3-layer architecture, where the system is divided into 3 layers.</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>CF_M01_AU14, CF_M01_AU15</t>
+          <t>CF_M01_P01</t>
         </is>
       </c>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr">
         <is>
-          <t>CF_M01_AU38</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>web socket, sql database</t>
-        </is>
-      </c>
+          <t>CF_M01_P02</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AU_35</t>
+          <t>AU_24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CF_M01_AU37</t>
+          <t>CF_M01_AU22</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D24" t="n">
         <v>1</v>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Kinesis Data Streams</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>The Web Socket service communicates with the Cloud Services.</t>
+          <t>Kinesis Data Streams és un servei de processament i ingesta de dades dirigit especialment al streaming de dades.</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>50</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>['AU_10', 'AU_12']</t>
+          <t>['AU_12']</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>AU_35</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>web socket, cloud services</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr"/>
+          <t>AU_24</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Kinesis Data Streams</t>
+        </is>
+      </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>The Web Socket service communicates with the Cloud Services.</t>
-        </is>
-      </c>
-      <c r="P24" t="n">
-        <v>42</v>
+          <t>Data processing and ingestion service aimed especially at data streaming. In the development of this project, Kinesis Data Streams has been used to transmit playlog and audit trail data.</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>50, 51</t>
+        </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CF_M01_AU14, CF_M01_AU16</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr">
         <is>
-          <t>CF_M01_AU37</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>web socket, aws cloud services set</t>
-        </is>
-      </c>
+          <t>CF_M01_AU22</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AU_36</t>
+          <t>P_01</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CF_M01_AU39</t>
+          <t>CF_M01_P01</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>pattern</t>
         </is>
       </c>
       <c r="D25" t="n">
         <v>1</v>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Client-Server</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Architectural Pattern</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>The Core service communicates with the Database.</t>
+          <t>En el nostre projecte la plataforma de Waapiti és un servei web que segueix l’arquitectura client-servidor.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>['AU_07', 'AU_11']</t>
-        </is>
-      </c>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>AU_36</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>core, database</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr"/>
+          <t>P_01</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Client-Server</t>
+        </is>
+      </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Architectural Pattern</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>The Core service communicates with the Database.</t>
+          <t>The Waapiti platform is a web service that follows the client-server architecture. In this type of architecture, the client is the one who makes requests to a server, which processes them and returns the response to the client.</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>42</v>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>CF_M01_AU11, CF_M01_AU15</t>
-        </is>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr">
         <is>
-          <t>CF_M01_AU39</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>core service, sql database</t>
-        </is>
-      </c>
+          <t>CF_M01_P01</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AU_37</t>
+          <t>AU_14</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CF_M01_AU40</t>
+          <t>CF_M01_AU18</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D26" t="n">
         <v>1</v>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Amazon DynamoDB</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>The Core service communicates with the Cloud Services.</t>
+          <t>DynamoDB: Aquest servei és una base de dades no relacional d’AWS.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>['AU_07', 'AU_12']</t>
+          <t>['AU_12']</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>AU_37</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>core, cloud services</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr"/>
+          <t>AU_14</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Amazon DynamoDB</t>
+        </is>
+      </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>The Core service communicates with the Cloud Services.</t>
+          <t>This service is a non-relational database from AWS. In our case, it is responsible for storing playlogs in real time.</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>CF_M01_AU11, CF_M01_AU16</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr">
         <is>
-          <t>CF_M01_AU40</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>core service, aws cloud services set</t>
-        </is>
-      </c>
+          <t>CF_M01_AU18</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AU_38</t>
+          <t>AU_16</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CF_M01_AU41</t>
+          <t>CF_M01_AU34</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D27" t="n">
         <v>1</v>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>TypeScript</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>The Analytical Module communicates with the Cloud Services.</t>
+          <t>Amb el llenguatge Typescript.</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>['AU_08', 'AU_12']</t>
+          <t>['AU_05']</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>AU_38</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>analytical module, cloud services</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr"/>
+          <t>AU_16</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>TypeScript</t>
+        </is>
+      </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>The Analytical Module communicates with the Cloud Services.</t>
+          <t>This programming language is built on top of JavaScript, it extends the JavaScript syntax.</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>CF_M01_AU12, CF_M01_AU16</t>
+          <t>CF_M01_AU33</t>
         </is>
       </c>
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr">
         <is>
-          <t>CF_M01_AU41</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>analytical module, aws cloud services set</t>
-        </is>
-      </c>
+          <t>CF_M01_AU34</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AU_40</t>
+          <t>AU_03</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CF_M01_AU33</t>
+          <t>CF_M01_AU07</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D28" t="n">
         <v>1</v>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Data Layer</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Layer</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>The Presentation Layer communicates with the Business Layer.</t>
+          <t>Capa de dades: És la capa que s’encarrega d'emmagatzemar totes les dades.</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -3291,65 +3321,61 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>['AU_01', 'AU_02']</t>
+          <t>['P_02']</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>AU_40</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>presentation layer, business layer</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr"/>
+          <t>AU_03</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Data Layer</t>
+        </is>
+      </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Layer</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>the presentation layer communicates with the business layer</t>
+          <t>It is the layer that is responsible for storing all the data. In our case, it would be the database and AWS storage services.</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>CF_M01_AU05, CF_M01_AU06</t>
+          <t>CF_M01_P02</t>
         </is>
       </c>
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr">
         <is>
-          <t>CF_M01_AU33</t>
-        </is>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>presentation layer, business layer</t>
-        </is>
-      </c>
+          <t>CF_M01_AU07</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>P_04</t>
+          <t>AU_25</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CF_M01_P04</t>
+          <t>CF_M01_AU23</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>pattern</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -3357,63 +3383,63 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>API Gateway</t>
+          <t>Kinesis Data Firehose</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Design Pattern</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>A design pattern that allows only one component to interact between users and the services provided by the platform, handling authorization and SSL.</t>
+          <t>El servei de Kinesis Data Firehose té com a funció principal la càrrega de grans quantitats de dades en magatzems de dades.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>51</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>['P_03']</t>
+          <t>['AU_12']</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>P_04</t>
+          <t>AU_25</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
-          <t>API Gateway</t>
+          <t>Kinesis Data Firehose</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Design Pattern</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>This design pattern allows only one component to interact between users and the services provided by the platform.</t>
+          <t>Its main function is to load large amounts of data into data warehouses. In this project we have used Kinesis Data Stream to store the playlogs and audit trail data in their corresponding S3 buckets. In addition, we have used one of the functionalities that Kinesis Data Firehose has with respect to the S3 service, which is dynamic partitioning.</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>CF_M01_P03</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr">
         <is>
-          <t>CF_M01_P04</t>
+          <t>CF_M01_AU23</t>
         </is>
       </c>
       <c r="T29" t="inlineStr"/>
@@ -3421,12 +3447,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AU_20</t>
+          <t>AU_21</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CF_M01_AU23</t>
+          <t>CF_M01_AU31</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3439,7 +3465,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Kinesis Data Firehose</t>
+          <t>TCP</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3449,29 +3475,29 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Service for loading streaming data into data stores.</t>
+          <t>La comunicació entre el servei de l’Api Gateway és mitjançant el protocol de comunicació TCP.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>['AU_12']</t>
+          <t>['AU_04']</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>AU_20</t>
+          <t>AU_21</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Kinesis Data Firehose</t>
+          <t>TCP</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3481,508 +3507,24 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Its main function is to load large amounts of data into data warehouses. In this project we have used Kinesis Data Stream to store the playlogs and audit trail data in their corresponding S3 buckets. In addition, we have used one of the functionalities that Kinesis Data Firehose has with respect to the S3 service, which is dynamic partitioning.</t>
+          <t>communication between the Api Gateway service is via the TCP communication protocol</t>
         </is>
       </c>
       <c r="P30" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_AU26,CF_M01_AU27</t>
         </is>
       </c>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr">
         <is>
-          <t>CF_M01_AU23</t>
+          <t>CF_M01_AU31</t>
         </is>
       </c>
       <c r="T30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>AU_18</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>CF_M01_AU21</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>AWS Glue</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Data integration and catalog service for metadata management.</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>49</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>['AU_12']</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>AU_18</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>AWS Glue</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>Serverless data integration service that allows us to detect, prepare, migrate and integrate data from different sources. In the case of the development of this project we have made use of the AWS Glue Data Catalog function. The use of this has been necessary to be able to store the metadata of the project data</t>
-        </is>
-      </c>
-      <c r="P31" t="n">
-        <v>49</v>
-      </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>CF_M01_AU16</t>
-        </is>
-      </c>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>CF_M01_AU21</t>
-        </is>
-      </c>
-      <c r="T31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>AU_08</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>CF_M01_AU12</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Analytical Module</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Service responsible for obtaining and processing playlogs, connections, and platform actions.</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>['AU_02']</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>AU_08</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>Analytical module</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>Its main function is to obtain and process data from playlogs, connections and platform actions. This service mainly interacts with cloud services, although it also interacts to a lesser extent with the database.</t>
-        </is>
-      </c>
-      <c r="P32" t="n">
-        <v>44</v>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>CF_M01_AU06</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>CF_M01_AU12</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>AU_03</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>CF_M01_AU07</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Data Layer</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Layer</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Layer responsible for storing all system data.</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>41, 44</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>AU_03</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>Data Layer</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>Layer</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>It is the layer that is responsible for storing all the data. In our case, it would be the database and AWS storage services.</t>
-        </is>
-      </c>
-      <c r="P33" t="n">
-        <v>41</v>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>CF_M01_P02</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>CF_M01_AU07</t>
-        </is>
-      </c>
-      <c r="T33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>AU_01</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>CF_M01_AU05</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Presentation Layer</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Layer</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Layer responsible for displaying information to the user, including web and mobile platforms.</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>41, 42</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>AU_01</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>Presentation Layer</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>Layer</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>It is the layer that is responsible for displaying information to the user. In this project, it is the visual interface of the Waapiti platform.</t>
-        </is>
-      </c>
-      <c r="P34" t="n">
-        <v>41</v>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>CF_M01_P02</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr">
-        <is>
-          <t>CF_M01_AU05</t>
-        </is>
-      </c>
-      <c r="T34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>AU_09</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>CF_M01_AU13</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>API Player</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Service responsible for communicating with players to receive status and content information.</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>['AU_02']</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>AU_09</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>Api Player</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>This service is responsible for communicating with the players, receiving all the information corresponding to them. The information they can receive can be the status of the player, the contents it plays, the schedules in which these contents should be played, etc. This information is processed and stored</t>
-        </is>
-      </c>
-      <c r="P35" t="n">
-        <v>44</v>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>CF_M01_AU06</t>
-        </is>
-      </c>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t>CF_M01_AU13</t>
-        </is>
-      </c>
-      <c r="T35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>AU_13</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>CF_M01_AU43</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>MySQL</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Database engine used for the relational database.</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>['AU_11']</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>AU_13</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>MySQL</t>
-        </is>
-      </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>As can be seen in Figure 9.1, the data layer is made up of AWS cloud services and the database. [...] The database used is a MySQL database that is responsible for storing all the data necessary for the operation of the system. This database is implemented in the RDS service [30], which is a distributed relational database service from AWS.</t>
-        </is>
-      </c>
-      <c r="P36" t="n">
-        <v>44</v>
-      </c>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t>CF_M01_AU15</t>
-        </is>
-      </c>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>CF_M01_AU43</t>
-        </is>
-      </c>
-      <c r="T36" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3995,7 +3537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4043,7 +3585,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AU_14</t>
+          <t>AU_11</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4059,79 +3601,79 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AWS service hosting the MySQL database.</t>
+          <t>Aquesta base de dades està implementada en el servei RDS, que és un servei de base de dades relacional distribuït d’AWS.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>CF_M01_AU17</t>
+          <t>CF_M01_AU18</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Amazon S3</t>
+          <t>Amazon DynamoDB</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0.6606</v>
+        <v>0.7803</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AU_21</t>
+          <t>AU_12</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>NestJS</t>
+          <t>Cloud Storage</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Backend framework used for developing microservices.</t>
+          <t>Conjunt de serveis cloud AWS: L’objectiu d’aquests serveis és formar un data lake on s’emmagatzemi tots els històrics.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>CF_M01_AU04</t>
+          <t>CF_M01_AU17</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>REST</t>
+          <t>Amazon S3</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.0762</v>
+        <v>0.7937</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AU_22</t>
+          <t>AU_27</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>TypeScript</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>presentation layer, api gateway</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Programming language used for development.</t>
+          <t>la capa de presentació es comunica amb la capa de negoci, més concretament amb l’Api Gateway, mitjançant el protocol HTTP.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -4139,159 +3681,155 @@
           <t>CF_M01_AU30</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Player</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>0.7845</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AU_24</t>
+          <t>AU_29</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>SAT</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>core, database, cloud storage</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Technical support department of Waapiti.</t>
+          <t>Servei Core: [...] Principalment, interactua amb la base de dades, encara que també interactua en menor mesura amb els serveis cloud.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>CF_M01_AU26</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>CF_M01_AU11</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Core Service</t>
+        </is>
+      </c>
       <c r="H5" t="n">
-        <v>0.0315</v>
+        <v>0.7564</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AU_25</t>
+          <t>AU_30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>analytical module, cloud storage, database</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Stakeholder responsible for product value and investment return.</t>
+          <t>Mòdul analític: [...] Principalment, aquest servei interactua amb els serveis cloud, encara que també interactua en menor mesura amb la base de dades.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>CF_M01_AU24</t>
+          <t>CF_M01_P01</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Internet</t>
+          <t>Client-Server</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.0336</v>
+        <v>0.6844</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AU_26</t>
+          <t>AU_32</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>web socket, player, database, cloud storage</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Author of the project responsible for design and implementation.</t>
+          <t>Web Socket: Aquest servei s’encarrega de realitzar la comunicació entre la plataforma i els players, i d’aquesta manera permet l’intercanvi d’informació entre ells. Processa les dades provinents dels players i les emmagatzema en la base de dades i en els serveis cloud.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CF_M01_AU30</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Player</t>
-        </is>
-      </c>
+          <t>CF_M01_AU29</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>0.0219</v>
+        <v>0.8249</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AU_27</t>
+          <t>AU_33</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>web socket, core, kinesis data firehose, cloud storage</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>External beneficiaries of the platform.</t>
+          <t>El microservei WebSocket [...] s’encarrega de rebre la informació dels players. Mentre que l’audit trail té com a generador el Core [...] Per part dels consumidors tenim el servei de Kinesis Data Firehose, que s’encarrega de guardar les dades en el S3.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>CF_M01_P01</t>
+          <t>CF_M01_AU23</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Client-Server</t>
+          <t>Kinesis Data Firehose</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>0.4629</v>
+        <v>0.7445000000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AU_39</t>
+          <t>AU_34</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4302,28 +3840,32 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>analytical module, database</t>
+          <t>amazon athena, amazon s3</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>The Analytical Module communicates with the Database.</t>
+          <t>El servei d’Amazon Athena és un servei que permet realitzar consultes en SQL sobre dades emmagatzemades en Amazon S3.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>CF_M01_AU42</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>CF_M01_AU17</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Amazon S3</t>
+        </is>
+      </c>
       <c r="H9" t="n">
-        <v>1</v>
+        <v>0.7753</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AU_41</t>
+          <t>AU_35</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4334,94 +3876,26 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>business layer, data layer</t>
+          <t>aws glue, amazon athena, amazon s3</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>The Business Layer communicates with the Data Layer.</t>
+          <t>El servei d’AWS Glue [...] treballa en conjunt amb Athena perquè pugui llegir les dades des del S3 de manera correcta.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>CF_M01_AU33</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
+          <t>CF_M01_AU21</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>AWS Glue</t>
+        </is>
+      </c>
       <c r="H10" t="n">
-        <v>0.745</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>P_03</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Architectural Pattern</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Microservices</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>The business and data layers are divided into several different services to improve security, scalability, and availability.</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>CF_M01_AU16</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>AWS cloud services set</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>0.261</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>P_05</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Design Pattern</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Data Lake</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>A centralized repository that allows for the storage of structured and unstructured data at any scale without needing to modify or structure it initially.</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>CF_M01_AU07</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Data Layer</t>
-        </is>
-      </c>
-      <c r="H12" t="n">
-        <v>0.4115</v>
+        <v>0.7893</v>
       </c>
     </row>
   </sheetData>
@@ -4435,7 +3909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4483,7 +3957,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CF_M01_AU01</t>
+          <t>CF_M01_AU02</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4493,86 +3967,86 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Server</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>The client is the user of the platform</t>
+          <t>The server is the software that is responsible for processing user requests.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>AU_23</t>
+          <t>P_01</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Player</t>
+          <t>Client-Server</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0.0234</v>
+        <v>0.8237</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CF_M01_AU02</t>
+          <t>CF_M01_AU24</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Connector</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Server</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>customer, server</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>The server is the software that is responsible for processing user requests.</t>
+          <t>Communication between the two components is carried out over the internet using the HTTP protocol and the REST API model.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>P_01</t>
+          <t>AU_20</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Client-Server</t>
+          <t>HTTP</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.5516</v>
+        <v>0.7941</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CF_M01_AU24</t>
+          <t>CF_M01_AU04</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Internet</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>customer, server</t>
-        </is>
-      </c>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>Communication between the two components is carried out over the internet using the HTTP protocol and the REST API model.</t>
@@ -4580,90 +4054,94 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>AU_30</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>AU_20</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>HTTP</t>
+        </is>
+      </c>
       <c r="H4" t="n">
-        <v>0.2176</v>
+        <v>0.6758999999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CF_M01_AU03</t>
+          <t>CF_M01_AU08</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>HTTP</t>
+          <t>Web platform interface</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Communication between the two components is carried out over the internet using the HTTP protocol and the REST API model.</t>
+          <t>In the case of this layer, you can see that it is made up of the interface of the web platform and the Waapiti mobile platform.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>AU_01</t>
+          <t>AU_20</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Presentation Layer</t>
+          <t>HTTP</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>0.7358</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CF_M01_AU04</t>
+          <t>CF_M01_AU09</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>REST</t>
+          <t>Waapiti Mobile Platform</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Communication between the two components is carried out over the internet using the HTTP protocol and the REST API model.</t>
+          <t>In the case of this layer, you can see that it is made up of the interface of the web platform and the Waapiti mobile platform.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AU_21</t>
+          <t>AU_04</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>NestJS</t>
+          <t>API Gateway</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.0762</v>
+        <v>0.6101</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CF_M01_AU25</t>
+          <t>CF_M01_AU30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4674,64 +4152,64 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>presentation layer, api gateway service</t>
+          <t>presentation layer, business layer</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>more specifically with the Api Gateway</t>
+          <t>the presentation layer communicates with the business layer</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>AU_06</t>
+          <t>AU_01</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>API Gateway</t>
+          <t>Presentation Layer</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0.5799</v>
+        <v>0.887</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CF_M01_AU34</t>
+          <t>CF_M01_AU29</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Connector</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>player, web socket</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>via the HTTP protocol</t>
+          <t>This service is responsible for communicating between the platform and the players.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AU_01</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Presentation Layer</t>
-        </is>
-      </c>
+          <t>AU_32</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>0.8249</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CF_M01_AU28</t>
+          <t>CF_M01_AU35</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4739,121 +4217,65 @@
           <t>Technology</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>AWSS RDS</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>communication between the Api Gateway service is via the TCP communication protocol</t>
+          <t>This database is implemented in the RDS service [30], which is a distributed relational database service from AWS.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>AU_01</t>
+          <t>AU_11</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Presentation Layer</t>
+          <t>Amazon RDS</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>0.742</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CF_M01_AU29</t>
+          <t>CF_M01_P03</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+          <t>Architectural Pattern</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Service-oriented</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>communication between the Api Gateway service is via the TCP communication protocol</t>
+          <t>Both the business layer and the data layer are divided into several different services</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>AU_01</t>
+          <t>P_01</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Presentation Layer</t>
+          <t>Client-Server</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>CF_M01_AU42</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Connector</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>core service, sql database</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>The Analytical Module communicates with the Database.</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>AU_39</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>CF_M01_P03</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Architectural Pattern</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Service-oriented</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Both the business layer and the data layer are divided into several different services</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>AU_37</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="n">
-        <v>0.2009</v>
+        <v>0.703</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
final prompts (compacted versions)
</commit_message>
<xml_diff>
--- a/outputs/evaluation/architecture/CF_M01_arch_eval.xlsx
+++ b/outputs/evaluation/architecture/CF_M01_arch_eval.xlsx
@@ -451,10 +451,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.7045</v>
+        <v>0.7317</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7949000000000001</v>
+        <v>0.7692</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -469,13 +469,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9286</v>
+        <v>0.9615</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7879</v>
+        <v>0.7576000000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9714</v>
+        <v>0.9722</v>
       </c>
     </row>
     <row r="6">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.931</v>
+        <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -517,10 +517,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.7931</v>
+        <v>0.931</v>
       </c>
       <c r="C8" t="n">
-        <v>0.8115</v>
+        <v>0.8635</v>
       </c>
     </row>
     <row r="9">
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.8276</v>
+        <v>0.8966</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.5385</v>
+        <v>0.8077</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -559,8 +559,10 @@
           <t>fixes</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>0</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -624,16 +626,16 @@
         <v>28</v>
       </c>
       <c r="C2" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8214</v>
+        <v>0.7857</v>
       </c>
     </row>
     <row r="3">
@@ -646,13 +648,13 @@
         <v>4</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
         <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="F3" t="n">
         <v>0.75</v>
@@ -668,13 +670,13 @@
         <v>7</v>
       </c>
       <c r="C4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D4" t="n">
         <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3125</v>
+        <v>0.3333</v>
       </c>
       <c r="F4" t="n">
         <v>0.7143</v>
@@ -723,7 +725,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
@@ -743,7 +745,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
@@ -754,7 +756,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>7 / 16</t>
+          <t>7 / 15</t>
         </is>
       </c>
     </row>
@@ -777,7 +779,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -797,7 +799,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.7045</v>
+        <v>0.7317</v>
       </c>
     </row>
     <row r="11">
@@ -807,7 +809,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.7949000000000001</v>
+        <v>0.7692</v>
       </c>
     </row>
     <row r="12">
@@ -886,19 +888,19 @@
         <v>33</v>
       </c>
       <c r="C2" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H2" t="n">
         <v>29</v>
@@ -914,7 +916,7 @@
         <v>38</v>
       </c>
       <c r="C3" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D3" t="n">
         <v>29</v>
@@ -926,7 +928,7 @@
         <v>29</v>
       </c>
       <c r="G3" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H3" t="n">
         <v>29</v>
@@ -942,7 +944,7 @@
         <v>38</v>
       </c>
       <c r="C4" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D4" t="n">
         <v>29</v>
@@ -954,7 +956,7 @@
         <v>29</v>
       </c>
       <c r="G4" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="H4" t="n">
         <v>29</v>
@@ -970,7 +972,7 @@
         <v>38</v>
       </c>
       <c r="C5" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D5" t="n">
         <v>29</v>
@@ -982,7 +984,7 @@
         <v>29</v>
       </c>
       <c r="G5" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H5" t="n">
         <v>29</v>
@@ -998,7 +1000,7 @@
         <v>36</v>
       </c>
       <c r="C6" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D6" t="n">
         <v>27</v>
@@ -1010,7 +1012,7 @@
         <v>26</v>
       </c>
       <c r="G6" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="H6" t="n">
         <v>29</v>
@@ -1026,13 +1028,13 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -1163,7 +1165,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AU_19</t>
+          <t>AU_01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1191,7 +1193,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>El client és l’usuari de la plataforma.</t>
+          <t>The client is the user of the platform.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1203,7 +1205,7 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>AU_19</t>
+          <t>AU_01</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
@@ -1241,12 +1243,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AU_17</t>
+          <t>AU_06</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_AU11</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1255,43 +1257,43 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.8603</v>
+        <v>0.8605</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Per la infraestructura es farà ús dels serveis cloud d’AWS.</t>
+          <t>This service is responsible for performing the business logic of the platform, it would be the main core of the platform.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>['AU_03']</t>
+          <t>['AU_03', 'P_04']</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>AU_17</t>
+          <t>AU_06</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>AWS cloud services set</t>
+          <t>Core Service</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -1301,23 +1303,21 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>As can be seen in Figure 9.1, the data layer is made up of AWS cloud services and the database. […] The objective of these services is to form a data lake where all the historical data is stored in order to process them in the analytical module.</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>44, 45</t>
-        </is>
+          <t>This service is responsible for carrying out the business logic of the platform, it would be the main core of the platform. Mainly, it interacts with the database, although it also interacts to a lesser extent with cloud services.</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>44</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>CF_M01_AU07</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_AU11</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
@@ -1325,12 +1325,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AU_05</t>
+          <t>AU_10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CF_M01_AU11</t>
+          <t>CF_M01_AU15</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1339,21 +1339,21 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.8605</v>
+        <v>0.8633</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Database</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Component</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Servei Core: Aquest servei s’encarrega de realitzar la lògica de negoci de la plataforma, seria el nucli principal de la plataforma.</t>
+          <t>The database used is a MySQL database that is responsible for storing all the data necessary for the operation of the system.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1363,29 +1363,29 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>['AU_02']</t>
+          <t>['AU_04']</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>AU_05</t>
+          <t>AU_10</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Core Service</t>
+          <t>SQL database</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Component</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>This service is responsible for carrying out the business logic of the platform, it would be the main core of the platform. Mainly, it interacts with the database, although it also interacts to a lesser extent with cloud services.</t>
+          <t>As can be seen in Figure 9.1, the data layer is made up of AWS cloud services and the database. [...] The database used is a MySQL database that is responsible for storing all the data necessary for the operation of the system. This database is implemented in the RDS service [30], which is a distributed relational database service from AWS.</t>
         </is>
       </c>
       <c r="P4" t="n">
@@ -1393,13 +1393,13 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_AU07</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>CF_M01_AU11</t>
+          <t>CF_M01_AU15</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
@@ -1407,12 +1407,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AU_09</t>
+          <t>AU_11</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CF_M01_AU15</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1421,11 +1421,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.8633</v>
+        <v>0.9241</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Database</t>
+          <t>AWS Cloud Services</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1435,43 +1435,45 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Base de dades: La base de dades utilitzada és una base de dades MySQL que s’encarrega d’emmagatzemar totes les dades necessàries per al funcionament del sistema.</t>
+          <t>The objective of these services is to form a data lake where all the history is stored to be able to process them in the analytical module.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>['AU_03']</t>
+          <t>['AU_04']</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>AU_09</t>
+          <t>AU_11</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>SQL database</t>
+          <t>AWS cloud services set</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>As can be seen in Figure 9.1, the data layer is made up of AWS cloud services and the database. [...] The database used is a MySQL database that is responsible for storing all the data necessary for the operation of the system. This database is implemented in the RDS service [30], which is a distributed relational database service from AWS.</t>
-        </is>
-      </c>
-      <c r="P5" t="n">
-        <v>44</v>
+          <t>As can be seen in Figure 9.1, the data layer is made up of AWS cloud services and the database. […] The objective of these services is to form a data lake where all the historical data is stored in order to process them in the analytical module.</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>44, 45</t>
+        </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -1481,7 +1483,7 @@
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
-          <t>CF_M01_AU15</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
@@ -1489,7 +1491,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AU_04</t>
+          <t>AU_05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1517,23 +1519,23 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>L’únic component que interactua de manera directa amb la capa de presentació és el mòdul Api Gateway.</t>
+          <t>This service is responsible for the management, authentication and authorization of platform users.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>43, 44</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>['P_03']</t>
+          <t>['AU_03', 'P_03', 'P_04']</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>AU_04</t>
+          <t>AU_05</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -1571,7 +1573,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AU_07</t>
+          <t>AU_08</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1599,7 +1601,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Api Player: Aquest servei s’encarrega de comunicar-se amb els players rebent tota la informació corresponent a aquest.</t>
+          <t>This service is responsible for communicating with the players receiving all the information corresponding to it.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1609,13 +1611,13 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>['AU_02']</t>
+          <t>['AU_03', 'P_04']</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>AU_07</t>
+          <t>AU_08</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
@@ -1653,12 +1655,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AU_06</t>
+          <t>AU_15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CF_M01_AU12</t>
+          <t>CF_M01_AU18</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1667,67 +1669,67 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.9891</v>
+        <v>0.9839</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Analytical Module</t>
+          <t>DynamoDB</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Mòdul analític: Aquest servei és el servei que s’ha començat a desenvolupar durant el desenvolupament d’aquest TFG.</t>
+          <t>This service is a non-relational database of AWS.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45, 48</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>['AU_02']</t>
+          <t>['AU_11']</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>AU_06</t>
+          <t>AU_15</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Analytical module</t>
+          <t>Amazon DynamoDB</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Its main function is to obtain and process data from playlogs, connections and platform actions. This service mainly interacts with cloud services, although it also interacts to a lesser extent with the database.</t>
+          <t>This service is a non-relational database from AWS. In our case, it is responsible for storing playlogs in real time.</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
         <is>
-          <t>CF_M01_AU12</t>
+          <t>CF_M01_AU18</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
@@ -1735,85 +1737,81 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P_03</t>
+          <t>AU_07</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CF_M01_P04</t>
+          <t>CF_M01_AU12</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>pattern</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>0.9891</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>API Gateway</t>
+          <t>Analytical Module</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Design Pattern</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Això és degut de què es segueix el patró de disseny de microserveis Api Gateway. Aquest patró de disseny permet que solament un component sigui qui interactuï entre els usuaris i els serveis que proporciona la plataforma.</t>
+          <t>This service is the service that has begun to be developed during the development of this TFG.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>['AU_02']</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>The document labels this as a 'patró de disseny de microserveis' (microservices design pattern). While it is a pattern used in microservices, it is classified here as a Design Pattern as per the provided definitions.</t>
-        </is>
-      </c>
+          <t>['AU_03', 'P_04']</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>P_03</t>
+          <t>AU_07</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>API Gateway</t>
+          <t>Analytical module</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Design Pattern</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>This design pattern allows only one component to interact between users and the services provided by the platform.</t>
+          <t>Its main function is to obtain and process data from playlogs, connections and platform actions. This service mainly interacts with cloud services, although it also interacts to a lesser extent with the database.</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>CF_M01_P03</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
-          <t>CF_M01_P04</t>
+          <t>CF_M01_AU12</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
@@ -1821,17 +1819,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AU_10</t>
+          <t>P_03</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CF_M01_AU32</t>
+          <t>CF_M01_P04</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>pattern</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1839,63 +1837,63 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>MySQL</t>
+          <t>API Gateway</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Design Pattern</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>La base de dades utilitzada és una base de dades MySQL.</t>
+          <t>Aquest patró de disseny permet que solament un component sigui qui interactuï entre els usuaris i els serveis que proporciona la plataforma.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>43</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>['AU_09']</t>
+          <t>['P_02', 'AU_05']</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>AU_10</t>
+          <t>P_03</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
-          <t>MySQL</t>
+          <t>API Gateway</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Design Pattern</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>The database used is a MySQL database that is responsible for storing all the data necessary for the operation of the system.</t>
+          <t>This design pattern allows only one component to interact between users and the services provided by the platform.</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>CF_M01_AU15</t>
+          <t>CF_M01_P03</t>
         </is>
       </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
-          <t>CF_M01_AU32</t>
+          <t>CF_M01_P04</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
@@ -1903,7 +1901,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AU_18</t>
+          <t>AU_22</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1931,7 +1929,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Un player consisteix en un dispositiu que pot ser intern o extern, que permet a les pantalles reproduir continguts.</t>
+          <t>A player consists of a device that can be internal or external, which allows screens to play content.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1943,7 +1941,7 @@
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>AU_18</t>
+          <t>AU_22</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -1977,7 +1975,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AU_22</t>
+          <t>AU_16</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2005,7 +2003,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>El servei d’Amazon Athena és un servei que permet realitzar consultes en SQL sobre dades emmagatzemades en Amazon S3.</t>
+          <t>The Amazon Athena service is a service that allows SQL queries to be performed on data stored in Amazon S3.</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -2015,13 +2013,13 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>['AU_12']</t>
+          <t>['AU_11']</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>AU_22</t>
+          <t>AU_16</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
@@ -2059,7 +2057,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AU_01</t>
+          <t>AU_02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2087,7 +2085,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Capa de presentació: És la capa que s’encarrega de mostrar la informació a l’usuari.</t>
+          <t>It is the layer that is responsible for displaying information to the user.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2103,7 +2101,7 @@
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>AU_01</t>
+          <t>AU_02</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -2169,17 +2167,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>La comunicació entre els dos components es realitza a través d’internet mitjançant el protocol HTTP.</t>
+          <t>Communication protocol used between the client and the server.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>41, 42</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>['AU_04']</t>
+          <t>['AU_02', 'AU_05']</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -2223,7 +2221,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AU_26</t>
+          <t>AU_23</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2247,28 +2245,28 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>L’únic component que interactua de manera directa amb la capa de presentació és el mòdul Api Gateway.</t>
+          <t>The presentation layer communicates with the business layer, more specifically with the Api Gateway, using the HTTP protocol.</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>42,43</t>
+          <t>42</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>['AU_04', 'AU_01']</t>
+          <t>['AU_02', 'AU_05']</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>AU_26</t>
+          <t>AU_23</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>api gateway, presentation layer</t>
+          <t>presentation layer, api gateway</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -2305,7 +2303,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AU_28</t>
+          <t>AU_24</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2329,7 +2327,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>El servei Api Gateway [...] processa les peticions per poder enviar-les al servei Core i al mòdul analític.</t>
+          <t>The Api Gateway processes requests to send them to the Core service and the analytical module.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2339,13 +2337,13 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>['AU_04', 'AU_05', 'AU_06']</t>
+          <t>['AU_05', 'AU_06', 'AU_07']</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>AU_28</t>
+          <t>AU_24</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2387,7 +2385,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AU_31</t>
+          <t>AU_28</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2411,7 +2409,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Api Player: Aquest servei s’encarrega de comunicar-se amb els players rebent tota la informació corresponent a aquest.</t>
+          <t>The Api Player communicates with players receiving all information corresponding to it. [...] This information is processed and stored.</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2421,13 +2419,13 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>['AU_07', 'AU_18']</t>
+          <t>['AU_08', 'AU_22']</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>AU_31</t>
+          <t>AU_28</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -2469,67 +2467,63 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AU_15</t>
+          <t>AU_29</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CF_M01_AU33</t>
+          <t>CF_M01_AU29</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="D18" t="n">
         <v>1</v>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>NestJS</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Connector</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Com a framework es farà ús de NestJS.</t>
+          <t>The Web Socket service is responsible for carrying out the communication between the platform and the players.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>['AU_05']</t>
+          <t>['AU_09', 'AU_22']</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>AU_15</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>NestJS</t>
-        </is>
-      </c>
+          <t>AU_29</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>web socket, player</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Connector</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>This framework is a NodeJS framework whose main function is to create backend applications. In this project, this framework has been used to develop the different services that interact with each other.</t>
+          <t>This service is responsible for communicating between the platform and the players.</t>
         </is>
       </c>
       <c r="P18" t="n">
@@ -2537,26 +2531,30 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>CF_M01_AU02</t>
+          <t>CF_M01_AU27, CF_M01_AU14</t>
         </is>
       </c>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
-          <t>CF_M01_AU33</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr"/>
+          <t>CF_M01_AU29</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>player, web socket</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AU_08</t>
+          <t>AU_12</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CF_M01_AU14</t>
+          <t>CF_M01_AU33</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2569,49 +2567,49 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Web Socket</t>
+          <t>NestJS</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Web Socket: Aquest servei s’encarrega de realitzar la comunicació entre la plataforma i els players, i d’aquesta manera permet l’intercanvi d’informació entre ells.</t>
+          <t>Framework used to develop the different services that interact with each other.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>46</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>['AU_02']</t>
+          <t>['AU_05', 'AU_06', 'AU_07', 'AU_08', 'AU_09']</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>AU_08</t>
+          <t>AU_12</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Web Socket</t>
+          <t>NestJS</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>This service is responsible for communicating between the platform and the players, thus allowing the exchange of information between them. It processes the data coming from the players and stores it in the database and in the cloud services.</t>
+          <t>This framework is a NodeJS framework whose main function is to create backend applications. In this project, this framework has been used to develop the different services that interact with each other.</t>
         </is>
       </c>
       <c r="P19" t="n">
@@ -2619,13 +2617,13 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_AU02</t>
         </is>
       </c>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr">
         <is>
-          <t>CF_M01_AU14</t>
+          <t>CF_M01_AU33</t>
         </is>
       </c>
       <c r="T19" t="inlineStr"/>
@@ -2633,12 +2631,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AU_13</t>
+          <t>AU_09</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CF_M01_AU17</t>
+          <t>CF_M01_AU14</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2651,63 +2649,63 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Amazon S3</t>
+          <t>Web Socket</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Amazon S3: Aquest és el servei d’emmagatzament d’objectes d’AWS.</t>
+          <t>This service is responsible for carrying out the communication between the platform and the players.</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>['AU_12']</t>
+          <t>['AU_03', 'P_04']</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>AU_13</t>
+          <t>AU_09</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Amazon S3</t>
+          <t>Web Socket</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>This is the AWS object storage service. In this project it is responsible for storing JSON documents containing playlogs, connections and audit trails.</t>
+          <t>This service is responsible for communicating between the platform and the players, thus allowing the exchange of information between them. It processes the data coming from the players and stores it in the database and in the cloud services.</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr">
         <is>
-          <t>CF_M01_AU17</t>
+          <t>CF_M01_AU14</t>
         </is>
       </c>
       <c r="T20" t="inlineStr"/>
@@ -2715,12 +2713,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AU_23</t>
+          <t>AU_14</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CF_M01_AU21</t>
+          <t>CF_M01_AU17</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2733,7 +2731,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>AWS Glue</t>
+          <t>Amazon S3</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2743,29 +2741,29 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>El servei d’AWS Glue és un servei d’integració de dades sense servidor.</t>
+          <t>This is the object storage service of AWS.</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>45, 48</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>['AU_12']</t>
+          <t>['AU_11']</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>AU_23</t>
+          <t>AU_14</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
-          <t>AWS Glue</t>
+          <t>Amazon S3</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2775,11 +2773,11 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Serverless data integration service that allows us to detect, prepare, migrate and integrate data from different sources. In the case of the development of this project we have made use of the AWS Glue Data Catalog function. The use of this has been necessary to be able to store the metadata of the project data</t>
+          <t>This is the AWS object storage service. In this project it is responsible for storing JSON documents containing playlogs, connections and audit trails.</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2789,7 +2787,7 @@
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr">
         <is>
-          <t>CF_M01_AU21</t>
+          <t>CF_M01_AU17</t>
         </is>
       </c>
       <c r="T21" t="inlineStr"/>
@@ -2797,12 +2795,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AU_02</t>
+          <t>AU_17</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_AU21</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2815,63 +2813,63 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Business Layer</t>
+          <t>AWS Glue</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Layer</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Capa de negoci: Aquesta capa és el nucli de l’aplicació, que s’encarrega de processar tota la informació.</t>
+          <t>The AWS Glue service is a serverless data integration service that allows us to detect, prepare, migrate and integrate data from different sources.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>49</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>['P_02']</t>
+          <t>['AU_11']</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>AU_02</t>
+          <t>AU_17</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Business Layer</t>
+          <t>AWS Glue</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Layer</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>This layer is the core of the application, which is responsible for processing all the information. In our context, it is the software that is responsible for processing user requests.</t>
+          <t>Serverless data integration service that allows us to detect, prepare, migrate and integrate data from different sources. In the case of the development of this project we have made use of the AWS Glue Data Catalog function. The use of this has been necessary to be able to store the metadata of the project data</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>CF_M01_P02</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_AU21</t>
         </is>
       </c>
       <c r="T22" t="inlineStr"/>
@@ -2879,17 +2877,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>P_02</t>
+          <t>AU_03</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CF_M01_P02</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>pattern</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -2897,17 +2895,17 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Three Layers</t>
+          <t>Business Layer</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Architectural Pattern</t>
+          <t>Layer</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Pel model client-servidor s’utilitza l’arquitectura de 3 capes, on el sistema es devidiex en 3 capes, la capa de presentació, la capa de negoci i la capa de dades.</t>
+          <t>This layer is the core of the application and is responsible for processing all the information.</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2917,29 +2915,29 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>['P_01']</t>
+          <t>['P_02']</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>P_02</t>
+          <t>AU_03</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Three Layers</t>
+          <t>Business Layer</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Architectural Pattern</t>
+          <t>Layer</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>The client-server model uses a 3-layer architecture, where the system is divided into 3 layers.</t>
+          <t>This layer is the core of the application, which is responsible for processing all the information. In our context, it is the software that is responsible for processing user requests.</t>
         </is>
       </c>
       <c r="P23" t="n">
@@ -2947,13 +2945,13 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>CF_M01_P01</t>
+          <t>CF_M01_P02</t>
         </is>
       </c>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr">
         <is>
-          <t>CF_M01_P02</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="T23" t="inlineStr"/>
@@ -2961,17 +2959,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AU_24</t>
+          <t>P_02</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CF_M01_AU22</t>
+          <t>CF_M01_P02</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>pattern</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -2979,65 +2977,63 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Kinesis Data Streams</t>
+          <t>Three Layers</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Architectural Pattern</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Kinesis Data Streams és un servei de processament i ingesta de dades dirigit especialment al streaming de dades.</t>
+          <t>Pel model client-servidor s’utilitza l’arquitectura de 3 capes, on el sistema es devidiex en 3 capes, la capa de presentació, la capa de negoci i la capa de dades.</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>['AU_12']</t>
+          <t>['P_01']</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>AU_24</t>
+          <t>P_02</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Kinesis Data Streams</t>
+          <t>Three Layers</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Architectural Pattern</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Data processing and ingestion service aimed especially at data streaming. In the development of this project, Kinesis Data Streams has been used to transmit playlog and audit trail data.</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>50, 51</t>
-        </is>
+          <t>The client-server model uses a 3-layer architecture, where the system is divided into 3 layers.</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>41</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_P01</t>
         </is>
       </c>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr">
         <is>
-          <t>CF_M01_AU22</t>
+          <t>CF_M01_P02</t>
         </is>
       </c>
       <c r="T24" t="inlineStr"/>
@@ -3045,17 +3041,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>P_01</t>
+          <t>AU_18</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CF_M01_P01</t>
+          <t>CF_M01_AU22</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>pattern</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -3063,55 +3059,65 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Client-Server</t>
+          <t>Kinesis Data Streams</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Architectural Pattern</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>En el nostre projecte la plataforma de Waapiti és un servei web que segueix l’arquitectura client-servidor.</t>
+          <t>Kinesis Data Streams is a data processing and ingestion service aimed especially at data streaming.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>41</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr"/>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>['AU_11']</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>P_01</t>
+          <t>AU_18</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Client-Server</t>
+          <t>Kinesis Data Streams</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Architectural Pattern</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>The Waapiti platform is a web service that follows the client-server architecture. In this type of architecture, the client is the one who makes requests to a server, which processes them and returns the response to the client.</t>
-        </is>
-      </c>
-      <c r="P25" t="n">
-        <v>41</v>
-      </c>
-      <c r="Q25" t="inlineStr"/>
+          <t>Data processing and ingestion service aimed especially at data streaming. In the development of this project, Kinesis Data Streams has been used to transmit playlog and audit trail data.</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>50, 51</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>CF_M01_AU16</t>
+        </is>
+      </c>
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr">
         <is>
-          <t>CF_M01_P01</t>
+          <t>CF_M01_AU22</t>
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
@@ -3119,17 +3125,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AU_14</t>
+          <t>P_01</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CF_M01_AU18</t>
+          <t>CF_M01_P01</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>pattern</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -3137,63 +3143,55 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Amazon DynamoDB</t>
+          <t>Client-Server</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Architectural Pattern</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>DynamoDB: Aquest servei és una base de dades no relacional d’AWS.</t>
+          <t>En el nostre projecte la plataforma de Waapiti és un servei web que segueix l’arquitectura client-servidor.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>['AU_12']</t>
-        </is>
-      </c>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>AU_14</t>
+          <t>P_01</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Amazon DynamoDB</t>
+          <t>Client-Server</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Architectural Pattern</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>This service is a non-relational database from AWS. In our case, it is responsible for storing playlogs in real time.</t>
+          <t>The Waapiti platform is a web service that follows the client-server architecture. In this type of architecture, the client is the one who makes requests to a server, which processes them and returns the response to the client.</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>45</v>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>CF_M01_AU16</t>
-        </is>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr">
         <is>
-          <t>CF_M01_AU18</t>
+          <t>CF_M01_P01</t>
         </is>
       </c>
       <c r="T26" t="inlineStr"/>
@@ -3201,7 +3199,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AU_16</t>
+          <t>AU_13</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3229,23 +3227,23 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Amb el llenguatge Typescript.</t>
+          <t>Programming language used for the development of the backend.</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>46</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>['AU_05']</t>
+          <t>['AU_12']</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>AU_16</t>
+          <t>AU_13</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
@@ -3283,7 +3281,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AU_03</t>
+          <t>AU_04</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3311,7 +3309,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Capa de dades: És la capa que s’encarrega d'emmagatzemar totes les dades.</t>
+          <t>It is the layer that is responsible for storing all the data.</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -3327,7 +3325,7 @@
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>AU_03</t>
+          <t>AU_04</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
@@ -3365,7 +3363,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AU_25</t>
+          <t>AU_19</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3393,7 +3391,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>El servei de Kinesis Data Firehose té com a funció principal la càrrega de grans quantitats de dades en magatzems de dades.</t>
+          <t>The Kinesis Data Firehose service has as its main function the loading of large amounts of data into data warehouses.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3403,13 +3401,13 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>['AU_12']</t>
+          <t>['AU_11']</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>AU_25</t>
+          <t>AU_19</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
@@ -3475,7 +3473,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>La comunicació entre el servei de l’Api Gateway és mitjançant el protocol de comunicació TCP.</t>
+          <t>Communication protocol used between the services.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3485,7 +3483,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>['AU_04']</t>
+          <t>['AU_03']</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -3537,7 +3535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3585,73 +3583,73 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AU_11</t>
+          <t>AU_25</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Amazon RDS</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>core, database, aws cloud services</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Aquesta base de dades està implementada en el servei RDS, que és un servei de base de dades relacional distribuït d’AWS.</t>
+          <t>The Core service interacts with the database, although it also interacts to a lesser extent with cloud services.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>CF_M01_AU18</t>
+          <t>CF_M01_AU11</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Amazon DynamoDB</t>
+          <t>Core Service</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0.7803</v>
+        <v>0.7699</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AU_12</t>
+          <t>AU_26</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Cloud Storage</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>analytical module, aws cloud services, database</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Conjunt de serveis cloud AWS: L’objectiu d’aquests serveis és formar un data lake on s’emmagatzemi tots els històrics.</t>
+          <t>The analytical module interacts with cloud services, although it also interacts to a lesser extent with the database.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>CF_M01_AU17</t>
+          <t>CF_M01_AU12</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Amazon S3</t>
+          <t>Analytical module</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.7937</v>
+        <v>0.7214</v>
       </c>
     </row>
     <row r="4">
@@ -3668,28 +3666,28 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>presentation layer, api gateway</t>
+          <t>web socket, database, aws cloud services</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>la capa de presentació es comunica amb la capa de negoci, més concretament amb l’Api Gateway, mitjançant el protocol HTTP.</t>
+          <t>The Web Socket service processes data from players and stores it in the database and cloud services.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>CF_M01_AU30</t>
+          <t>CF_M01_AU29</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>0.7845</v>
+        <v>0.799</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AU_29</t>
+          <t>AU_30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3700,32 +3698,32 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>core, database, cloud storage</t>
+          <t>kinesis data streams, web socket, core</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Servei Core: [...] Principalment, interactua amb la base de dades, encara que també interactua en menor mesura amb els serveis cloud.</t>
+          <t>Kinesis Data Streams reads data from different generators (Producers) and sends them to the consumers. [...] In the case of playlogs the generator is the WebSocket microservice. [...] While the audit trail has as a generator the Core.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>CF_M01_AU11</t>
+          <t>CF_M01_AU22</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Core Service</t>
+          <t>Kinesis Data Streams</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.7564</v>
+        <v>0.7364000000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AU_30</t>
+          <t>AU_31</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3736,26 +3734,26 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>analytical module, cloud storage, database</t>
+          <t>kinesis data firehose, aws cloud services</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Mòdul analític: [...] Principalment, aquest servei interactua amb els serveis cloud, encara que també interactua en menor mesura amb la base de dades.</t>
+          <t>For the consumers we have the Kinesis Data Firehose service, which is responsible for saving the data in S3.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>CF_M01_P01</t>
+          <t>CF_M01_AU23</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Client-Server</t>
+          <t>Kinesis Data Firehose</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.6844</v>
+        <v>0.8252</v>
       </c>
     </row>
     <row r="7">
@@ -3772,22 +3770,26 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>web socket, player, database, cloud storage</t>
+          <t>analytical module, amazon athena</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Web Socket: Aquest servei s’encarrega de realitzar la comunicació entre la plataforma i els players, i d’aquesta manera permet l’intercanvi d’informació entre ells. Processa les dades provinents dels players i les emmagatzema en la base de dades i en els serveis cloud.</t>
+          <t>The analytical module uses the AWS Athena service to perform queries on data stored in Amazon S3.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CF_M01_AU29</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>CF_M01_AU17</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Amazon S3</t>
+        </is>
+      </c>
       <c r="H7" t="n">
-        <v>0.8249</v>
+        <v>0.7654</v>
       </c>
     </row>
     <row r="8">
@@ -3804,98 +3806,62 @@
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>web socket, core, kinesis data firehose, cloud storage</t>
+          <t>analytical module, database</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>El microservei WebSocket [...] s’encarrega de rebre la informació dels players. Mentre que l’audit trail té com a generador el Core [...] Per part dels consumidors tenim el servei de Kinesis Data Firehose, que s’encarrega de guardar les dades en el S3.</t>
+          <t>The analytical module also has the database service, which is responsible for connecting and performing queries to the platform's database.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>CF_M01_AU23</t>
+          <t>CF_M01_AU12</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Kinesis Data Firehose</t>
+          <t>Analytical module</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>0.7445000000000001</v>
+        <v>0.7284</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AU_34</t>
+          <t>P_04</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Connector</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>amazon athena, amazon s3</t>
-        </is>
-      </c>
+          <t>Architectural Pattern</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Microservices</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>El servei d’Amazon Athena és un servei que permet realitzar consultes en SQL sobre dades emmagatzemades en Amazon S3.</t>
+          <t>L’objectiu d’això és millorar la seguretat, l’escalabilitat i la disponibilitat del sistema... les diferents capes que formen el sistema es componen de diversos serveis que interactuen entre si.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>CF_M01_AU17</t>
+          <t>CF_M01_AU10</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Amazon S3</t>
+          <t>API Gateway Service</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0.7753</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>AU_35</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Connector</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>aws glue, amazon athena, amazon s3</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>El servei d’AWS Glue [...] treballa en conjunt amb Athena perquè pugui llegir les dades des del S3 de manera correcta.</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>CF_M01_AU21</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>AWS Glue</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>0.7893</v>
+        <v>0.7454</v>
       </c>
     </row>
   </sheetData>
@@ -4018,16 +3984,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>AU_20</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>HTTP</t>
-        </is>
-      </c>
+          <t>AU_23</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>0.7941</v>
+        <v>0.823</v>
       </c>
     </row>
     <row r="4">
@@ -4126,7 +4088,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AU_04</t>
+          <t>AU_05</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -4162,7 +4124,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>AU_01</t>
+          <t>AU_02</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4177,33 +4139,37 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CF_M01_AU29</t>
+          <t>CF_M01_AU32</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Connector</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>player, web socket</t>
-        </is>
-      </c>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MySQL</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>This service is responsible for communicating between the platform and the players.</t>
+          <t>The database used is a MySQL database that is responsible for storing all the data necessary for the operation of the system.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AU_32</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+          <t>AU_10</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
       <c r="H8" t="n">
-        <v>0.8249</v>
+        <v>0.7872</v>
       </c>
     </row>
     <row r="9">
@@ -4235,11 +4201,11 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Amazon RDS</t>
+          <t>AWS Cloud Services</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0.742</v>
+        <v>0.658</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Finish experimentation for requirement v2
</commit_message>
<xml_diff>
--- a/outputs/evaluation/architecture/CF_M01_arch_eval.xlsx
+++ b/outputs/evaluation/architecture/CF_M01_arch_eval.xlsx
@@ -451,10 +451,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6415</v>
+        <v>0.7174</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8718</v>
+        <v>0.8462</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -469,13 +469,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8529</v>
+        <v>0.9032</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8788</v>
+        <v>0.8485</v>
       </c>
       <c r="D3" t="n">
-        <v>0.957</v>
+        <v>0.9626</v>
       </c>
     </row>
     <row r="6">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.7188</v>
+        <v>0.875</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -517,10 +517,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.9062</v>
+        <v>0.9375</v>
       </c>
       <c r="C8" t="n">
-        <v>0.8764</v>
+        <v>0.8823</v>
       </c>
     </row>
     <row r="9">
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.6153999999999999</v>
+        <v>0.6333</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -559,10 +559,8 @@
           <t>fixes</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B11" t="n">
+        <v>0</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -626,16 +624,16 @@
         <v>28</v>
       </c>
       <c r="C2" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E2" t="n">
-        <v>0.8667</v>
+        <v>0.9258999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9286</v>
+        <v>0.8929</v>
       </c>
     </row>
     <row r="3">
@@ -670,13 +668,13 @@
         <v>7</v>
       </c>
       <c r="C4" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D4" t="n">
         <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2632</v>
+        <v>0.3333</v>
       </c>
       <c r="F4" t="n">
         <v>0.7143</v>
@@ -725,7 +723,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4">
@@ -745,7 +743,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6">
@@ -756,7 +754,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>7 / 19</t>
+          <t>7 / 15</t>
         </is>
       </c>
     </row>
@@ -779,7 +777,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -799,7 +797,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.6415</v>
+        <v>0.7174</v>
       </c>
     </row>
     <row r="11">
@@ -809,7 +807,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.8718</v>
+        <v>0.8462</v>
       </c>
     </row>
     <row r="12">
@@ -888,19 +886,19 @@
         <v>33</v>
       </c>
       <c r="C2" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H2" t="n">
         <v>32</v>
@@ -916,7 +914,7 @@
         <v>38</v>
       </c>
       <c r="C3" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D3" t="n">
         <v>32</v>
@@ -928,7 +926,7 @@
         <v>32</v>
       </c>
       <c r="G3" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="H3" t="n">
         <v>32</v>
@@ -944,7 +942,7 @@
         <v>38</v>
       </c>
       <c r="C4" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D4" t="n">
         <v>32</v>
@@ -956,7 +954,7 @@
         <v>32</v>
       </c>
       <c r="G4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H4" t="n">
         <v>32</v>
@@ -972,7 +970,7 @@
         <v>38</v>
       </c>
       <c r="C5" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D5" t="n">
         <v>32</v>
@@ -984,7 +982,7 @@
         <v>32</v>
       </c>
       <c r="G5" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H5" t="n">
         <v>32</v>
@@ -1000,19 +998,19 @@
         <v>36</v>
       </c>
       <c r="C6" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D6" t="n">
         <v>30</v>
       </c>
       <c r="E6" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F6" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G6" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="H6" t="n">
         <v>32</v>
@@ -1028,13 +1026,13 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -1165,12 +1163,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AU_14</t>
+          <t>AU_06</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CF_M01_AU35</t>
+          <t>CF_M01_AU09</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1179,67 +1177,67 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.7771</v>
+        <v>0.7532</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AWS RDS</t>
+          <t>Mobile Platform Interface</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Component</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>This database is implemented in the RDS service, which is a distributed relational database service from AWS.</t>
+          <t>In the case of this layer, it can be observed that it is formed by the web platform interface and the mobile platform of Waapiti.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>42</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>['AU_12']</t>
+          <t>['AU_02']</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>AU_14</t>
+          <t>AU_06</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>AWSS RDS</t>
+          <t>Waapiti Mobile Platform</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>This database is implemented in the RDS service [30], which is a distributed relational database service from AWS.</t>
+          <t>In the case of this layer, you can see that it is made up of the interface of the web platform and the Waapiti mobile platform.</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>CF_M01_AU15</t>
+          <t>CF_M01_AU05</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>CF_M01_AU35</t>
+          <t>CF_M01_AU09</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
@@ -1247,12 +1245,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AU_06</t>
+          <t>AU_14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CF_M01_AU09</t>
+          <t>CF_M01_AU35</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1261,67 +1259,67 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.8012</v>
+        <v>0.7771</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Mobile Platform</t>
+          <t>AWS RDS</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>In the case of this layer, it can be observed that it is formed by the web platform interface and the Waapiti mobile platform.</t>
+          <t>This database is implemented in the RDS service, which is a distributed relational database service from AWS.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>45</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>['AU_02']</t>
+          <t>['AU_12']</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>AU_06</t>
+          <t>AU_14</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Waapiti Mobile Platform</t>
+          <t>AWSS RDS</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>In the case of this layer, you can see that it is made up of the interface of the web platform and the Waapiti mobile platform.</t>
+          <t>This database is implemented in the RDS service [30], which is a distributed relational database service from AWS.</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>CF_M01_AU05</t>
+          <t>CF_M01_AU15</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>CF_M01_AU09</t>
+          <t>CF_M01_AU35</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
@@ -1343,11 +1341,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.8139</v>
+        <v>0.8514</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Database Service</t>
+          <t>Relational Database</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1416,7 +1414,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CF_M01_AU04</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1425,11 +1423,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.8436</v>
+        <v>0.8603</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>REST API</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1439,15 +1437,19 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The communication between the two components is carried out through the internet using the REST API model.</t>
+          <t>For the infrastructure, the cloud services of AWS will be used.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>41</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>['AU_04']</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
@@ -1457,31 +1459,33 @@
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>REST</t>
+          <t>AWS cloud services set</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Communication between the two components is carried out over the internet using the HTTP protocol and the REST API model.</t>
-        </is>
-      </c>
-      <c r="P5" t="n">
-        <v>41</v>
+          <t>As can be seen in Figure 9.1, the data layer is made up of AWS cloud services and the database. […] The objective of these services is to form a data lake where all the historical data is stored in order to process them in the analytical module.</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>44, 45</t>
+        </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>CF_M01_AU24</t>
+          <t>CF_M01_AU07</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
-          <t>CF_M01_AU04</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
@@ -1489,12 +1493,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AU_20</t>
+          <t>AU_08</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_AU11</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1503,39 +1507,43 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.8603</v>
+        <v>0.8605</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>For the infrastructure, the cloud services of AWS will be used.</t>
+          <t>This service is responsible for performing the business logic of the platform, it would be the main core of the platform.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>['AU_03']</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>AU_20</t>
+          <t>AU_08</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>AWS cloud services set</t>
+          <t>Core Service</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1545,23 +1553,21 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>As can be seen in Figure 9.1, the data layer is made up of AWS cloud services and the database. […] The objective of these services is to form a data lake where all the historical data is stored in order to process them in the analytical module.</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>44, 45</t>
-        </is>
+          <t>This service is responsible for carrying out the business logic of the platform, it would be the main core of the platform. Mainly, it interacts with the database, although it also interacts to a lesser extent with cloud services.</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>44</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>CF_M01_AU07</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_AU11</t>
         </is>
       </c>
       <c r="T6" t="inlineStr"/>
@@ -1569,12 +1575,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AU_08</t>
+          <t>AU_07</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CF_M01_AU11</t>
+          <t>CF_M01_AU10</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1583,21 +1589,21 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.8605</v>
+        <v>0.9471000000000001</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>API Gateway</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>This service is responsible for performing the business logic of the platform, it would be the main core of the platform.</t>
+          <t>This service is responsible for the management, authentication and authorization of platform users.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1607,19 +1613,19 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>['AU_03', 'P_04']</t>
+          <t>['AU_03', 'P_03']</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>AU_08</t>
+          <t>AU_07</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Core Service</t>
+          <t>API Gateway Service</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1629,7 +1635,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>This service is responsible for carrying out the business logic of the platform, it would be the main core of the platform. Mainly, it interacts with the database, although it also interacts to a lesser extent with cloud services.</t>
+          <t>This service is responsible for the management, authentication and authorization of platform users. It defines all the REST API routes and processes the requests to be sent to the Core service and the analytical module.</t>
         </is>
       </c>
       <c r="P7" t="n">
@@ -1643,7 +1649,7 @@
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
-          <t>CF_M01_AU11</t>
+          <t>CF_M01_AU10</t>
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
@@ -1651,12 +1657,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AU_05</t>
+          <t>AU_10</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CF_M01_AU08</t>
+          <t>CF_M01_AU13</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1665,43 +1671,43 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.9185</v>
+        <v>0.9573</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Web Platform</t>
+          <t>API Player</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>In the case of this layer, it can be observed that it is formed by the web platform interface and the Waapiti mobile platform.</t>
+          <t>This service is responsible for communicating with the players receiving all the information corresponding to it.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>['AU_02']</t>
+          <t>['AU_03']</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>AU_05</t>
+          <t>AU_10</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Web platform interface</t>
+          <t>Api Player</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1711,21 +1717,21 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>In the case of this layer, you can see that it is made up of the interface of the web platform and the Waapiti mobile platform.</t>
+          <t>This service is responsible for communicating with the players, receiving all the information corresponding to them. The information they can receive can be the status of the player, the contents it plays, the schedules in which these contents should be played, etc. This information is processed and stored</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>CF_M01_AU05</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
         <is>
-          <t>CF_M01_AU08</t>
+          <t>CF_M01_AU13</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
@@ -1733,12 +1739,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AU_07</t>
+          <t>AU_05</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CF_M01_AU10</t>
+          <t>CF_M01_AU08</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1747,11 +1753,11 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.9471000000000001</v>
+        <v>0.9715</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>API Gateway</t>
+          <t>Web Platform Interface</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1761,29 +1767,29 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The only component that interacts directly with the presentation layer is the Api Gateway module.</t>
+          <t>In the case of this layer, it can be observed that it is formed by the web platform interface and the mobile platform of Waapiti.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>42</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>['AU_03', 'P_03']</t>
+          <t>['AU_02']</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>AU_07</t>
+          <t>AU_05</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>API Gateway Service</t>
+          <t>Web platform interface</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1793,21 +1799,21 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>This service is responsible for the management, authentication and authorization of platform users. It defines all the REST API routes and processes the requests to be sent to the Core service and the analytical module.</t>
+          <t>In the case of this layer, you can see that it is made up of the interface of the web platform and the Waapiti mobile platform.</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_AU05</t>
         </is>
       </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
-          <t>CF_M01_AU10</t>
+          <t>CF_M01_AU08</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
@@ -1815,12 +1821,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AU_10</t>
+          <t>AU_17</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CF_M01_AU13</t>
+          <t>CF_M01_AU18</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1829,67 +1835,67 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.9573</v>
+        <v>0.9839</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>API Player</t>
+          <t>DynamoDB</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>This service is responsible for communicating with the players by receiving all the information corresponding to it.</t>
+          <t>This service is a non-relational database from AWS.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>['AU_03']</t>
+          <t>['AU_15']</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>AU_10</t>
+          <t>AU_17</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Api Player</t>
+          <t>Amazon DynamoDB</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>This service is responsible for communicating with the players, receiving all the information corresponding to them. The information they can receive can be the status of the player, the contents it plays, the schedules in which these contents should be played, etc. This information is processed and stored</t>
+          <t>This service is a non-relational database from AWS. In our case, it is responsible for storing playlogs in real time.</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
-          <t>CF_M01_AU13</t>
+          <t>CF_M01_AU18</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
@@ -1897,12 +1903,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AU_17</t>
+          <t>AU_09</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CF_M01_AU18</t>
+          <t>CF_M01_AU12</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1911,67 +1917,67 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.9839</v>
+        <v>0.9891</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>DynamoDB</t>
+          <t>Analytical Module</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>This service is a non-relational database of AWS.</t>
+          <t>The analytical module has as its main function to obtain and process the data of the playlogs, the connections and the actions in the platform.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>['AU_15']</t>
+          <t>['AU_03']</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>AU_17</t>
+          <t>AU_09</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Amazon DynamoDB</t>
+          <t>Analytical module</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>This service is a non-relational database from AWS. In our case, it is responsible for storing playlogs in real time.</t>
+          <t>Its main function is to obtain and process data from playlogs, connections and platform actions. This service mainly interacts with cloud services, although it also interacts to a lesser extent with the database.</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr">
         <is>
-          <t>CF_M01_AU18</t>
+          <t>CF_M01_AU12</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
@@ -1979,81 +1985,85 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AU_09</t>
+          <t>P_03</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CF_M01_AU12</t>
+          <t>CF_M01_P04</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>pattern</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.9891</v>
+        <v>1</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Analytical Module</t>
+          <t>API Gateway</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Design Pattern</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The analytical module has as its main function to obtain and process the data of the playlogs, the connections and the actions in the platform.</t>
+          <t>Això és degut de què es segueix el patró de disseny de microserveis Api Gateway.</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>43</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>['AU_03', 'P_04']</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
+          <t>['AU_07']</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>The document labels it as a 'patró de disseny de microserveis' (microservices design pattern), but API Gateway is a well-known design pattern. I have classified it as a Design Pattern.</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>AU_09</t>
+          <t>P_03</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Analytical module</t>
+          <t>API Gateway</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Design Pattern</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Its main function is to obtain and process data from playlogs, connections and platform actions. This service mainly interacts with cloud services, although it also interacts to a lesser extent with the database.</t>
+          <t>This design pattern allows only one component to interact between users and the services provided by the platform.</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_P03</t>
         </is>
       </c>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
-          <t>CF_M01_AU12</t>
+          <t>CF_M01_P04</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
@@ -2061,17 +2071,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>P_03</t>
+          <t>AU_13</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CF_M01_P04</t>
+          <t>CF_M01_AU32</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>pattern</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -2079,63 +2089,63 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>API Gateway</t>
+          <t>MySQL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Design Pattern</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Això és degut de què es segueix el patró de disseny de microserveis Api Gateway.</t>
+          <t>The database used is a MySQL database.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>['P_02', 'AU_07']</t>
+          <t>['AU_12']</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>P_03</t>
+          <t>AU_13</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>API Gateway</t>
+          <t>MySQL</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Design Pattern</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>This design pattern allows only one component to interact between users and the services provided by the platform.</t>
+          <t>The database used is a MySQL database that is responsible for storing all the data necessary for the operation of the system.</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>CF_M01_P03</t>
+          <t>CF_M01_AU15</t>
         </is>
       </c>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
-          <t>CF_M01_P04</t>
+          <t>CF_M01_AU32</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
@@ -2143,12 +2153,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AU_13</t>
+          <t>AU_27</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CF_M01_AU32</t>
+          <t>CF_M01_AU27</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2161,63 +2171,55 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MySQL</t>
+          <t>Player</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The database used is a MySQL database.</t>
+          <t>A player consists of a device that can be internal or external, which allows the screens to play content.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>['AU_12']</t>
-        </is>
-      </c>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>AU_13</t>
+          <t>AU_27</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
-          <t>MySQL</t>
+          <t>Player</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>The database used is a MySQL database that is responsible for storing all the data necessary for the operation of the system.</t>
+          <t>A player consists of a device that can be internal or external, which allows screens to reproduce content on the screens.</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>44</v>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>CF_M01_AU15</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
-          <t>CF_M01_AU32</t>
+          <t>CF_M01_AU27</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
@@ -2225,12 +2227,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AU_30</t>
+          <t>AU_23</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CF_M01_AU27</t>
+          <t>CF_M01_AU20</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2243,55 +2245,63 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Player</t>
+          <t>Amazon Athena</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>A player consists of a device that can be internal or external, which allows the screens to play content.</t>
+          <t>The Amazon Athena service is a service that allows SQL queries to be performed on data stored in Amazon S3.</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>['AU_09']</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>AU_30</t>
+          <t>AU_23</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Player</t>
+          <t>Amazon Athena</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>A player consists of a device that can be internal or external, which allows screens to reproduce content on the screens.</t>
+          <t>Service that allows you to perform SQL queries on data stored in Amazon S3</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q15" t="inlineStr"/>
+        <v>49</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>CF_M01_AU16</t>
+        </is>
+      </c>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
-          <t>CF_M01_AU27</t>
+          <t>CF_M01_AU20</t>
         </is>
       </c>
       <c r="T15" t="inlineStr"/>
@@ -2299,12 +2309,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AU_24</t>
+          <t>AU_02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CF_M01_AU20</t>
+          <t>CF_M01_AU05</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2317,63 +2327,63 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Amazon Athena</t>
+          <t>Presentation Layer</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Layer</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>The Amazon Athena service is a service that allows SQL queries to be performed on data stored in Amazon S3.</t>
+          <t>It is the layer that is responsible for displaying information to the user.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>['AU_15']</t>
+          <t>['P_02']</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>AU_24</t>
+          <t>AU_02</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Amazon Athena</t>
+          <t>Presentation Layer</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Layer</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Service that allows you to perform SQL queries on data stored in Amazon S3</t>
+          <t>It is the layer that is responsible for displaying information to the user. In this project, it is the visual interface of the Waapiti platform.</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_P02</t>
         </is>
       </c>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr">
         <is>
-          <t>CF_M01_AU20</t>
+          <t>CF_M01_AU05</t>
         </is>
       </c>
       <c r="T16" t="inlineStr"/>
@@ -2381,12 +2391,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AU_02</t>
+          <t>AU_18</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CF_M01_AU05</t>
+          <t>CF_M01_AU03</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2399,17 +2409,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Presentation Layer</t>
+          <t>HTTP</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Layer</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>It is the layer that is responsible for displaying information to the user.</t>
+          <t>The communication between the two components is carried out through the internet using the HTTP protocol.</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2419,29 +2429,29 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>['P_02']</t>
+          <t>['AU_07']</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>AU_02</t>
+          <t>AU_18</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Presentation Layer</t>
+          <t>HTTP</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Layer</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>It is the layer that is responsible for displaying information to the user. In this project, it is the visual interface of the Waapiti platform.</t>
+          <t>Communication between the two components is carried out over the internet using the HTTP protocol and the REST API model.</t>
         </is>
       </c>
       <c r="P17" t="n">
@@ -2449,13 +2459,13 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>CF_M01_P02</t>
+          <t>CF_M01_AU24, CF_M01_AU25</t>
         </is>
       </c>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr">
         <is>
-          <t>CF_M01_AU05</t>
+          <t>CF_M01_AU03</t>
         </is>
       </c>
       <c r="T17" t="inlineStr"/>
@@ -2463,90 +2473,94 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AU_21</t>
+          <t>AU_28</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CF_M01_AU03</t>
+          <t>CF_M01_AU25</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="D18" t="n">
         <v>1</v>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>HTTP</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Connector</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>The communication between the two components is carried out through the internet using the HTTP protocol.</t>
+          <t>The presentation layer communicates with the business layer, more specifically with the Api Gateway, through the HTTP protocol.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>41</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr"/>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>['AU_02', 'AU_07']</t>
+        </is>
+      </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>AU_21</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>HTTP</t>
-        </is>
-      </c>
+          <t>AU_28</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>presentation layer, api gateway</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Connector</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Communication between the two components is carried out over the internet using the HTTP protocol and the REST API model.</t>
+          <t>the presentation layer communicates with the business layer more specifically with the Api Gateway</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>CF_M01_AU24, CF_M01_AU25</t>
+          <t>CF_M01_AU05, CF_M01_AU10</t>
         </is>
       </c>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
-          <t>CF_M01_AU03</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr"/>
+          <t>CF_M01_AU25</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>presentation layer, api gateway service</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AU_31</t>
+          <t>AU_29</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CF_M01_AU25</t>
+          <t>CF_M01_AU26</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2565,28 +2579,28 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>The presentation layer communicates with the business layer, more specifically with the Api Gateway, using the HTTP protocol.</t>
+          <t>The Api Gateway service processes requests to be able to send them to the Core service and the analytical module.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>['AU_02', 'AU_07']</t>
+          <t>['AU_07', 'AU_08', 'AU_09']</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>AU_31</t>
+          <t>AU_29</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>presentation layer, api gateway</t>
+          <t>api gateway, core, analytical module</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -2597,38 +2611,38 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>the presentation layer communicates with the business layer more specifically with the Api Gateway</t>
+          <t>Furthermore, it can be observed that three components are directly or indirectly related to the presentation layer, that is, they interact with users. These components would be, the Api Gateway, the Core and the analytical module. […] the only component that interacts directly with the presentation layer is the Api Gateway module [...]</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>CF_M01_AU05, CF_M01_AU10</t>
+          <t>CF_M01_AU10, CF_M01_AU11, CF_M01_AU12</t>
         </is>
       </c>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr">
         <is>
-          <t>CF_M01_AU25</t>
+          <t>CF_M01_AU26</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>presentation layer, api gateway service</t>
+          <t>api gateway service, core service, analytical module</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AU_32</t>
+          <t>AU_33</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CF_M01_AU26</t>
+          <t>CF_M01_AU29</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2647,7 +2661,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>The Api Gateway service processes requests to send them to the Core service and the Analytical Module.</t>
+          <t>The Web Socket service carries out the communication between the platform and the players.</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2657,18 +2671,18 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>['AU_07', 'AU_08', 'AU_09']</t>
+          <t>['AU_11', 'AU_27']</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>AU_32</t>
+          <t>AU_33</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>api gateway, core, analytical module</t>
+          <t>web socket, player</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -2679,33 +2693,33 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Furthermore, it can be observed that three components are directly or indirectly related to the presentation layer, that is, they interact with users. These components would be, the Api Gateway, the Core and the analytical module. […] the only component that interacts directly with the presentation layer is the Api Gateway module [...]</t>
+          <t>This service is responsible for communicating between the platform and the players.</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>CF_M01_AU10, CF_M01_AU11, CF_M01_AU12</t>
+          <t>CF_M01_AU27, CF_M01_AU14</t>
         </is>
       </c>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr">
         <is>
-          <t>CF_M01_AU26</t>
+          <t>CF_M01_AU29</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>api gateway service, core service, analytical module</t>
+          <t>player, web socket</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AU_36</t>
+          <t>AU_34</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2729,7 +2743,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>The Api Player service is responsible for communicating with the players by receiving all the information corresponding to it. [...] This information is processed and stored.</t>
+          <t>The Api Player service communicates with the players receiving all the information corresponding to it.</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2739,13 +2753,13 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>['AU_10', 'AU_30']</t>
+          <t>['AU_10', 'AU_27']</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>AU_36</t>
+          <t>AU_34</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2787,7 +2801,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AU_18</t>
+          <t>AU_20</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2831,7 +2845,7 @@
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>AU_18</t>
+          <t>AU_20</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
@@ -2892,7 +2906,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3033,7 +3047,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AU_25</t>
+          <t>AU_24</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3071,13 +3085,13 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>['AU_15']</t>
+          <t>['AU_09']</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>AU_25</t>
+          <t>AU_24</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
@@ -3279,7 +3293,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AU_26</t>
+          <t>AU_25</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3317,13 +3331,13 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>['AU_15']</t>
+          <t>['AU_08']</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>AU_26</t>
+          <t>AU_25</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
@@ -3437,7 +3451,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AU_19</t>
+          <t>AU_21</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3465,7 +3479,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>With the Typescript language.</t>
+          <t>With the language Typescript.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3475,13 +3489,13 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>['AU_03']</t>
+          <t>['AU_20']</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>AU_19</t>
+          <t>AU_21</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
@@ -3601,7 +3615,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AU_27</t>
+          <t>AU_26</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3639,13 +3653,13 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>['AU_15']</t>
+          <t>['AU_08']</t>
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
-          <t>AU_27</t>
+          <t>AU_26</t>
         </is>
       </c>
       <c r="L32" t="inlineStr"/>
@@ -3683,7 +3697,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AU_23</t>
+          <t>AU_19</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3711,7 +3725,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>The communication between the Api Gateway service is through the TCP communication protocol.</t>
+          <t>The communication between the API Gateway service is through the TCP communication protocol.</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3719,11 +3733,15 @@
           <t>44</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>['AU_07']</t>
+        </is>
+      </c>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
-          <t>AU_23</t>
+          <t>AU_19</t>
         </is>
       </c>
       <c r="L33" t="inlineStr"/>
@@ -3769,7 +3787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3863,7 +3881,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Data Lake Service</t>
+          <t>Data Lake</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -3883,85 +3901,85 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.7272999999999999</v>
+        <v>0.7526</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AU_28</t>
+          <t>AU_30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>AWS CDK</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>core, relational database</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AWS Cloud Development, also called AWS CDK, is the AWS framework that allows the construction of cloud applications.</t>
+          <t>The Core service interacts with the database, although it also interacts to a lesser extent with cloud services.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>CF_M01_AU18</t>
+          <t>CF_M01_AU11</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Amazon DynamoDB</t>
+          <t>Core Service</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0.7153</v>
+        <v>0.7699</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AU_29</t>
+          <t>AU_31</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>AWS CloudFormation</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>analytical module, data lake</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AWS CloudFormation is an Amazon service that helps configure AWS resources.</t>
+          <t>The analytical module interacts with cloud services, although it also interacts to a lesser extent with the database.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_AU12</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>AWS cloud services set</t>
+          <t>Analytical module</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.7708</v>
+        <v>0.7214</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AU_33</t>
+          <t>AU_32</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3972,32 +3990,28 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>api gateway, core, analytical module</t>
+          <t>web socket, relational database, data lake</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>The communication between the Api Gateway service is through the TCP communication protocol.</t>
+          <t>The Web Socket service processes data from players and stores it in the database and cloud services.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>CF_M01_AU10</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>API Gateway Service</t>
-        </is>
-      </c>
+          <t>CF_M01_AU29</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>0.8048999999999999</v>
+        <v>0.799</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AU_34</t>
+          <t>AU_35</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4008,32 +4022,32 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>core, database service, aws</t>
+          <t>analytical module, amazon athena, amazon s3</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>The Core service interacts with the database, although it also interacts to a lesser extent with cloud services.</t>
+          <t>The analytical module uses Amazon Athena to perform queries on data stored in Amazon S3.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CF_M01_AU11</t>
+          <t>CF_M01_AU17</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Core Service</t>
+          <t>Amazon S3</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0.7699</v>
+        <v>0.7788</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AU_35</t>
+          <t>AU_36</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4044,26 +4058,26 @@
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>analytical module, aws, database service</t>
+          <t>core, web socket, kinesis data streams</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>The Analytical Module interacts with cloud services, although it also interacts to a lesser extent with the database.</t>
+          <t>The microservices (Core and Web Socket) send data to the Kinesis Data Stream.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>CF_M01_AU12</t>
+          <t>CF_M01_AU22</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Analytical module</t>
+          <t>Kinesis Data Streams</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>0.7204</v>
+        <v>0.7889</v>
       </c>
     </row>
     <row r="9">
@@ -4080,202 +4094,62 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>web socket, player, database service, aws</t>
+          <t>kinesis data firehose, kinesis data streams, amazon s3</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>The Web Socket service is responsible for carrying out the communication between the platform and the players, and in this way allows the exchange of information between them. [...] It processes the data coming from the players and stores them in the database and in the cloud services.</t>
+          <t>Kinesis Data Firehose reads from the Kinesis Data Stream and saves the data in Amazon S3.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>CF_M01_AU29</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>CF_M01_AU23</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Kinesis Data Firehose</t>
+        </is>
+      </c>
       <c r="H9" t="n">
-        <v>0.8564000000000001</v>
+        <v>0.8948</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AU_38</t>
+          <t>P_04</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Connector</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>analytical module, amazon athena, amazon s3</t>
-        </is>
-      </c>
+          <t>Design Pattern</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Data lake</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>The Analytical Module uses the Amazon Athena service to perform queries on data stored in Amazon S3.</t>
+          <t>Un data lake consisteix en un dipòsit de dades que poden ser emmagatzemades en el seu format natural.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>CF_M01_AU17</t>
+          <t>CF_M01_AU07</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Amazon S3</t>
+          <t>Data Layer</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0.7613</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>AU_39</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Connector</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>aws glue, amazon athena, amazon s3</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>The AWS Glue service works in conjunction with Athena so that it can read data from S3 correctly.</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>CF_M01_AU21</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>AWS Glue</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>0.8133</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>AU_40</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Connector</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>kinesis data streams, web socket, core</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Kinesis Data Streams reads data from different generators (Producers) and sends them to the consumers (Consumers). [...] In the case of the playlogs the generator is the WebSocket microservice [...] while the audit trail has as generator the Core.</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>CF_M01_AU22</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Kinesis Data Streams</t>
-        </is>
-      </c>
-      <c r="H12" t="n">
-        <v>0.7433999999999999</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>AU_41</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Connector</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>kinesis data firehose, kinesis data streams, amazon s3</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>For the consumers we have the Kinesis Data Firehose service, which is responsible for saving the data in the S3.</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>CF_M01_AU23</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Kinesis Data Firehose</t>
-        </is>
-      </c>
-      <c r="H13" t="n">
-        <v>0.8238</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>P_04</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Architectural Pattern</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Microservices</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>En el cas de la plataforma de Waapiti, l’arquitectura física no es correspon exactament a l’arquitectura lògica, ja que tant la capa de negoci com la capa de dades es divideixen en diversos serveis diferents.</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>CF_M01_AU10</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>API Gateway Service</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>0.7454</v>
+        <v>0.7534</v>
       </c>
     </row>
   </sheetData>
@@ -4434,54 +4308,54 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>AU_31</t>
+          <t>AU_28</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>0.823</v>
+        <v>0.8183</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CF_M01_AU30</t>
+          <t>CF_M01_AU04</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Connector</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>presentation layer, business layer</t>
-        </is>
-      </c>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>the presentation layer communicates with the business layer</t>
+          <t>Communication between the two components is carried out over the internet using the HTTP protocol and the REST API model.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>AU_02</t>
+          <t>AU_18</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Presentation Layer</t>
+          <t>HTTP</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.887</v>
+        <v>0.6758999999999999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CF_M01_AU29</t>
+          <t>CF_M01_AU30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4492,22 +4366,26 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>player, web socket</t>
+          <t>presentation layer, business layer</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>This service is responsible for communicating between the platform and the players.</t>
+          <t>the presentation layer communicates with the business layer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AU_37</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>AU_02</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Presentation Layer</t>
+        </is>
+      </c>
       <c r="H6" t="n">
-        <v>0.8564000000000001</v>
+        <v>0.887</v>
       </c>
     </row>
     <row r="7">
@@ -4534,16 +4412,16 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>AU_12</t>
+          <t>P_01</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Database Service</t>
+          <t>Client-Server</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0.7045</v>
+        <v>0.703</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement architecture extraction till v3
</commit_message>
<xml_diff>
--- a/outputs/evaluation/architecture/CF_M01_arch_eval.xlsx
+++ b/outputs/evaluation/architecture/CF_M01_arch_eval.xlsx
@@ -451,10 +451,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.7174</v>
+        <v>0.7692</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8462</v>
+        <v>0.7692</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -469,13 +469,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9032</v>
+        <v>0.8182</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8485</v>
+        <v>0.8438</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9626</v>
+        <v>0.9691</v>
       </c>
     </row>
     <row r="6">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.875</v>
+        <v>0.931</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -517,10 +517,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.9375</v>
+        <v>0.931</v>
       </c>
       <c r="C8" t="n">
-        <v>0.8823</v>
+        <v>0.8772</v>
       </c>
     </row>
     <row r="9">
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.875</v>
+        <v>0.8966</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.6333</v>
+        <v>0.7778</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -556,7 +556,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>fixes</t>
+          <t>fixedType</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -624,16 +624,16 @@
         <v>28</v>
       </c>
       <c r="C2" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9258999999999999</v>
+        <v>0.8276</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8929</v>
+        <v>0.8571</v>
       </c>
     </row>
     <row r="3">
@@ -668,16 +668,16 @@
         <v>7</v>
       </c>
       <c r="C4" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3333</v>
+        <v>0.5</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7143</v>
+        <v>0.4286</v>
       </c>
     </row>
   </sheetData>
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
@@ -754,7 +754,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>7 / 15</t>
+          <t>7 / 6</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>5 / 5</t>
+          <t>3 / 3</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.7174</v>
+        <v>0.7692</v>
       </c>
     </row>
     <row r="11">
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.8462</v>
+        <v>0.7692</v>
       </c>
     </row>
     <row r="12">
@@ -883,25 +883,25 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>32</v>
+      </c>
+      <c r="C2" t="n">
         <v>33</v>
       </c>
-      <c r="C2" t="n">
-        <v>31</v>
-      </c>
       <c r="D2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H2" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3">
@@ -914,22 +914,22 @@
         <v>38</v>
       </c>
       <c r="C3" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D3" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E3" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F3" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G3" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H3" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -942,22 +942,22 @@
         <v>38</v>
       </c>
       <c r="C4" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D4" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E4" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F4" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G4" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H4" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
@@ -970,22 +970,22 @@
         <v>38</v>
       </c>
       <c r="C5" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D5" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E5" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F5" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G5" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H5" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6">
@@ -998,35 +998,35 @@
         <v>36</v>
       </c>
       <c r="C6" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D6" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E6" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F6" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G6" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H6" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>fixes</t>
+          <t>fixedType</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -1041,7 +1041,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1055,7 +1055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T33"/>
+  <dimension ref="A1:T30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>LLM_fixes</t>
+          <t>LLM_fixedType</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>GT_fixes</t>
+          <t>GT_fixedType</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>In the case of this layer, it can be observed that it is formed by the web platform interface and the mobile platform of Waapiti.</t>
+          <t>In the case of this layer, it is formed by the web platform interface and the mobile platform of Waapiti.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1245,12 +1245,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AU_14</t>
+          <t>AU_18</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CF_M01_AU35</t>
+          <t>CF_M01_AU04</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1259,11 +1259,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.7771</v>
+        <v>0.8436</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AWS RDS</t>
+          <t>REST API</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1273,29 +1273,29 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>This database is implemented in the RDS service, which is a distributed relational database service from AWS.</t>
+          <t>The communication between the two components is carried out through the internet using the REST API model.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>['AU_12']</t>
+          <t>['AU_03', 'AU_30']</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>AU_14</t>
+          <t>AU_18</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>AWSS RDS</t>
+          <t>REST</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -1305,21 +1305,21 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>This database is implemented in the RDS service [30], which is a distributed relational database service from AWS.</t>
+          <t>Communication between the two components is carried out over the internet using the HTTP protocol and the REST API model.</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>CF_M01_AU15</t>
+          <t>CF_M01_AU24</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>CF_M01_AU35</t>
+          <t>CF_M01_AU04</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
@@ -1341,16 +1341,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.8514</v>
+        <v>0.8633</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Relational Database</t>
+          <t>Database</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Component</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>['AU_04']</t>
+          <t>['AU_04', 'P_04']</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -1409,12 +1409,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AU_22</t>
+          <t>AU_10</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_AU13</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1423,43 +1423,43 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.8603</v>
+        <v>0.8889</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Player API Service</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>For the infrastructure, the cloud services of AWS will be used.</t>
+          <t>This service is responsible for communicating with the players receiving all the information corresponding to it.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>['AU_04']</t>
+          <t>['AU_03', 'P_04']</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>AU_22</t>
+          <t>AU_10</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>AWS cloud services set</t>
+          <t>Api Player</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -1469,23 +1469,21 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>As can be seen in Figure 9.1, the data layer is made up of AWS cloud services and the database. […] The objective of these services is to form a data lake where all the historical data is stored in order to process them in the analytical module.</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>44, 45</t>
-        </is>
+          <t>This service is responsible for communicating with the players, receiving all the information corresponding to them. The information they can receive can be the status of the player, the contents it plays, the schedules in which these contents should be played, etc. This information is processed and stored</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>44</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>CF_M01_AU07</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_AU13</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
@@ -1493,12 +1491,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AU_08</t>
+          <t>AU_13</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CF_M01_AU11</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1507,11 +1505,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.8605</v>
+        <v>0.9241</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>AWS Cloud Services</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1521,29 +1519,29 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>This service is responsible for performing the business logic of the platform, it would be the main core of the platform.</t>
+          <t>The objective of these services is to form a data lake where all the history is stored to be able to process them in the analytical module.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>['AU_03']</t>
+          <t>['AU_04']</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>AU_08</t>
+          <t>AU_13</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Core Service</t>
+          <t>AWS cloud services set</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1553,21 +1551,23 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>This service is responsible for carrying out the business logic of the platform, it would be the main core of the platform. Mainly, it interacts with the database, although it also interacts to a lesser extent with cloud services.</t>
-        </is>
-      </c>
-      <c r="P6" t="n">
-        <v>44</v>
+          <t>As can be seen in Figure 9.1, the data layer is made up of AWS cloud services and the database. […] The objective of these services is to form a data lake where all the historical data is stored in order to process them in the analytical module.</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>44, 45</t>
+        </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_AU07</t>
         </is>
       </c>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">
         <is>
-          <t>CF_M01_AU11</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="T6" t="inlineStr"/>
@@ -1575,12 +1575,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AU_07</t>
+          <t>AU_11</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CF_M01_AU10</t>
+          <t>CF_M01_AU14</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1589,11 +1589,11 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.9471000000000001</v>
+        <v>0.9483</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>API Gateway</t>
+          <t>Web Socket Service</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>This service is responsible for the management, authentication and authorization of platform users.</t>
+          <t>This service is responsible for carrying out the communication between the platform and the players.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1613,19 +1613,19 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>['AU_03', 'P_03']</t>
+          <t>['AU_03', 'P_04']</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>AU_07</t>
+          <t>AU_11</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>API Gateway Service</t>
+          <t>Web Socket</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>This service is responsible for the management, authentication and authorization of platform users. It defines all the REST API routes and processes the requests to be sent to the Core service and the analytical module.</t>
+          <t>This service is responsible for communicating between the platform and the players, thus allowing the exchange of information between them. It processes the data coming from the players and stores it in the database and in the cloud services.</t>
         </is>
       </c>
       <c r="P7" t="n">
@@ -1649,7 +1649,7 @@
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
-          <t>CF_M01_AU10</t>
+          <t>CF_M01_AU14</t>
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
@@ -1657,12 +1657,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AU_10</t>
+          <t>AU_05</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CF_M01_AU13</t>
+          <t>CF_M01_AU08</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1671,43 +1671,43 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.9573</v>
+        <v>0.9715</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>API Player</t>
+          <t>Web Platform Interface</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Component</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>This service is responsible for communicating with the players receiving all the information corresponding to it.</t>
+          <t>In the case of this layer, it is formed by the web platform interface and the mobile platform of Waapiti.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>42</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>['AU_03']</t>
+          <t>['AU_02']</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>AU_10</t>
+          <t>AU_05</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Api Player</t>
+          <t>Web platform interface</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1717,21 +1717,21 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>This service is responsible for communicating with the players, receiving all the information corresponding to them. The information they can receive can be the status of the player, the contents it plays, the schedules in which these contents should be played, etc. This information is processed and stored</t>
+          <t>In the case of this layer, you can see that it is made up of the interface of the web platform and the Waapiti mobile platform.</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_AU05</t>
         </is>
       </c>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
         <is>
-          <t>CF_M01_AU13</t>
+          <t>CF_M01_AU08</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AU_05</t>
+          <t>AU_23</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CF_M01_AU08</t>
+          <t>CF_M01_AU18</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1753,67 +1753,67 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.9715</v>
+        <v>0.9839</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Web Platform Interface</t>
+          <t>DynamoDB</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>In the case of this layer, it can be observed that it is formed by the web platform interface and the mobile platform of Waapiti.</t>
+          <t>This service is a non-relational database of AWS.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>45</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>['AU_02']</t>
+          <t>['AU_13']</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>AU_05</t>
+          <t>AU_23</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Web platform interface</t>
+          <t>Amazon DynamoDB</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>In the case of this layer, you can see that it is made up of the interface of the web platform and the Waapiti mobile platform.</t>
+          <t>This service is a non-relational database from AWS. In our case, it is responsible for storing playlogs in real time.</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>CF_M01_AU05</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
-          <t>CF_M01_AU08</t>
+          <t>CF_M01_AU18</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
@@ -1821,12 +1821,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AU_17</t>
+          <t>AU_09</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CF_M01_AU18</t>
+          <t>CF_M01_AU12</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1835,67 +1835,67 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.9839</v>
+        <v>0.9891</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>DynamoDB</t>
+          <t>Analytical Module</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>This service is a non-relational database from AWS.</t>
+          <t>The analytical module has as its main function to obtain and process the data of the playlogs, the connections and the actions in platform.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>['AU_15']</t>
+          <t>['AU_03', 'P_04']</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>AU_17</t>
+          <t>AU_09</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Amazon DynamoDB</t>
+          <t>Analytical module</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>This service is a non-relational database from AWS. In our case, it is responsible for storing playlogs in real time.</t>
+          <t>Its main function is to obtain and process data from playlogs, connections and platform actions. This service mainly interacts with cloud services, although it also interacts to a lesser extent with the database.</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
-          <t>CF_M01_AU18</t>
+          <t>CF_M01_AU12</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
@@ -1903,81 +1903,81 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AU_09</t>
+          <t>P_03</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CF_M01_AU12</t>
+          <t>CF_M01_P04</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>pattern</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.9891</v>
+        <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Analytical Module</t>
+          <t>API Gateway</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Design Pattern</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The analytical module has as its main function to obtain and process the data of the playlogs, the connections and the actions in the platform.</t>
+          <t>Això és degut de què es segueix el patró de disseny de microserveis Api Gateway.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>['AU_03']</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>The document labels it as a 'patró de disseny de microserveis', but it is a well-known design pattern used to manage service interaction.</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>AU_09</t>
+          <t>P_03</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Analytical module</t>
+          <t>API Gateway</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Design Pattern</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Its main function is to obtain and process data from playlogs, connections and platform actions. This service mainly interacts with cloud services, although it also interacts to a lesser extent with the database.</t>
+          <t>This design pattern allows only one component to interact between users and the services provided by the platform.</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_P03</t>
         </is>
       </c>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr">
         <is>
-          <t>CF_M01_AU12</t>
+          <t>CF_M01_P04</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
@@ -1985,17 +1985,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>P_03</t>
+          <t>AU_20</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CF_M01_P04</t>
+          <t>CF_M01_AU32</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>pattern</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -2003,67 +2003,63 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>API Gateway</t>
+          <t>MySQL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Design Pattern</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Això és degut de què es segueix el patró de disseny de microserveis Api Gateway.</t>
+          <t>The database used is a MySQL database.</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>['AU_07']</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>The document labels it as a 'patró de disseny de microserveis' (microservices design pattern), but API Gateway is a well-known design pattern. I have classified it as a Design Pattern.</t>
-        </is>
-      </c>
+          <t>['AU_12']</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>P_03</t>
+          <t>AU_20</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
-          <t>API Gateway</t>
+          <t>MySQL</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Design Pattern</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>This design pattern allows only one component to interact between users and the services provided by the platform.</t>
+          <t>The database used is a MySQL database that is responsible for storing all the data necessary for the operation of the system.</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>CF_M01_P03</t>
+          <t>CF_M01_AU15</t>
         </is>
       </c>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
-          <t>CF_M01_P04</t>
+          <t>CF_M01_AU32</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
@@ -2071,12 +2067,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AU_13</t>
+          <t>AU_24</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CF_M01_AU32</t>
+          <t>CF_M01_AU20</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2089,7 +2085,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MySQL</t>
+          <t>Amazon Athena</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2099,29 +2095,29 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The database used is a MySQL database.</t>
+          <t>The Amazon Athena service is a service that allows SQL queries to be performed on data stored in Amazon S3.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>49</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>['AU_12']</t>
+          <t>['AU_13']</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>AU_13</t>
+          <t>AU_24</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>MySQL</t>
+          <t>Amazon Athena</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -2131,21 +2127,21 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>The database used is a MySQL database that is responsible for storing all the data necessary for the operation of the system.</t>
+          <t>Service that allows you to perform SQL queries on data stored in Amazon S3</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>CF_M01_AU15</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
-          <t>CF_M01_AU32</t>
+          <t>CF_M01_AU20</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
@@ -2153,12 +2149,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AU_27</t>
+          <t>AU_02</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CF_M01_AU27</t>
+          <t>CF_M01_AU05</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2171,55 +2167,63 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Player</t>
+          <t>Presentation Layer</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Layer</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>A player consists of a device that can be internal or external, which allows the screens to play content.</t>
+          <t>It is the layer that is responsible for displaying information to the user.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>['P_02']</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>AU_27</t>
+          <t>AU_02</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Player</t>
+          <t>Presentation Layer</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Layer</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>A player consists of a device that can be internal or external, which allows screens to reproduce content on the screens.</t>
+          <t>It is the layer that is responsible for displaying information to the user. In this project, it is the visual interface of the Waapiti platform.</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q14" t="inlineStr"/>
+        <v>41</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>CF_M01_P02</t>
+        </is>
+      </c>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
-          <t>CF_M01_AU27</t>
+          <t>CF_M01_AU05</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
@@ -2227,12 +2231,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AU_23</t>
+          <t>AU_08</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CF_M01_AU20</t>
+          <t>CF_M01_AU11</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2245,63 +2249,63 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Amazon Athena</t>
+          <t>Core Service</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>The Amazon Athena service is a service that allows SQL queries to be performed on data stored in Amazon S3.</t>
+          <t>This service is responsible for performing the business logic of the platform, it would be the main core of the platform.</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>['AU_09']</t>
+          <t>['AU_03', 'P_04']</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>AU_23</t>
+          <t>AU_08</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Amazon Athena</t>
+          <t>Core Service</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Service that allows you to perform SQL queries on data stored in Amazon S3</t>
+          <t>This service is responsible for carrying out the business logic of the platform, it would be the main core of the platform. Mainly, it interacts with the database, although it also interacts to a lesser extent with cloud services.</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
-          <t>CF_M01_AU20</t>
+          <t>CF_M01_AU11</t>
         </is>
       </c>
       <c r="T15" t="inlineStr"/>
@@ -2309,12 +2313,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AU_02</t>
+          <t>AU_17</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CF_M01_AU05</t>
+          <t>CF_M01_AU03</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2327,17 +2331,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Presentation Layer</t>
+          <t>HTTP</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Layer</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>It is the layer that is responsible for displaying information to the user.</t>
+          <t>The communication between the two components is carried out through the internet using the HTTP protocol.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2347,29 +2351,29 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>['P_02']</t>
+          <t>['AU_03', 'AU_30']</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>AU_02</t>
+          <t>AU_17</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Presentation Layer</t>
+          <t>HTTP</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Layer</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>It is the layer that is responsible for displaying information to the user. In this project, it is the visual interface of the Waapiti platform.</t>
+          <t>Communication between the two components is carried out over the internet using the HTTP protocol and the REST API model.</t>
         </is>
       </c>
       <c r="P16" t="n">
@@ -2377,13 +2381,13 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>CF_M01_P02</t>
+          <t>CF_M01_AU24, CF_M01_AU25</t>
         </is>
       </c>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr">
         <is>
-          <t>CF_M01_AU05</t>
+          <t>CF_M01_AU03</t>
         </is>
       </c>
       <c r="T16" t="inlineStr"/>
@@ -2391,94 +2395,94 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AU_18</t>
+          <t>AU_30</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CF_M01_AU03</t>
+          <t>CF_M01_AU25</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="D17" t="n">
         <v>1</v>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>HTTP</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Connector</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>The communication between the two components is carried out through the internet using the HTTP protocol.</t>
+          <t>La capa de presentació es comunica amb la capa de negoci, més concretament amb l’Api Gateway, mitjançant el protocol HTTP.</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>['AU_07']</t>
+          <t>['AU_02', 'AU_07']</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>AU_18</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>HTTP</t>
-        </is>
-      </c>
+          <t>AU_30</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>presentation layer, api gateway service</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Connector</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Communication between the two components is carried out over the internet using the HTTP protocol and the REST API model.</t>
+          <t>the presentation layer communicates with the business layer more specifically with the Api Gateway</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>CF_M01_AU24, CF_M01_AU25</t>
+          <t>CF_M01_AU05, CF_M01_AU10</t>
         </is>
       </c>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr">
         <is>
-          <t>CF_M01_AU03</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr"/>
+          <t>CF_M01_AU25</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>presentation layer, api gateway service</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AU_28</t>
+          <t>AU_31</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CF_M01_AU25</t>
+          <t>CF_M01_AU26</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2497,28 +2501,28 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>The presentation layer communicates with the business layer, more specifically with the Api Gateway, through the HTTP protocol.</t>
+          <t>La comunicació entre el servei de l’Api Gateway és mitjançant el protocol de comunicació TCP.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>['AU_02', 'AU_07']</t>
+          <t>['AU_07', 'AU_08', 'AU_09']</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>AU_28</t>
+          <t>AU_31</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>presentation layer, api gateway</t>
+          <t>api gateway service, core service, analytical module</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -2529,139 +2533,143 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>the presentation layer communicates with the business layer more specifically with the Api Gateway</t>
+          <t>Furthermore, it can be observed that three components are directly or indirectly related to the presentation layer, that is, they interact with users. These components would be, the Api Gateway, the Core and the analytical module. […] the only component that interacts directly with the presentation layer is the Api Gateway module [...]</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>CF_M01_AU05, CF_M01_AU10</t>
+          <t>CF_M01_AU10, CF_M01_AU11, CF_M01_AU12</t>
         </is>
       </c>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
-          <t>CF_M01_AU25</t>
+          <t>CF_M01_AU26</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>presentation layer, api gateway service</t>
+          <t>api gateway service, core service, analytical module</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AU_29</t>
+          <t>AU_14</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CF_M01_AU26</t>
+          <t>CF_M01_AU33</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D19" t="n">
         <v>1</v>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>NestJS</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>The Api Gateway service processes requests to be able to send them to the Core service and the analytical module.</t>
+          <t>As a framework, NestJS will be used.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>['AU_07', 'AU_08', 'AU_09']</t>
+          <t>['AU_03']</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>AU_29</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>api gateway, core, analytical module</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr"/>
+          <t>AU_14</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>NestJS</t>
+        </is>
+      </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Furthermore, it can be observed that three components are directly or indirectly related to the presentation layer, that is, they interact with users. These components would be, the Api Gateway, the Core and the analytical module. […] the only component that interacts directly with the presentation layer is the Api Gateway module [...]</t>
+          <t>This framework is a NodeJS framework whose main function is to create backend applications. In this project, this framework has been used to develop the different services that interact with each other.</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>CF_M01_AU10, CF_M01_AU11, CF_M01_AU12</t>
+          <t>CF_M01_AU02</t>
         </is>
       </c>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr">
         <is>
-          <t>CF_M01_AU26</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>api gateway service, core service, analytical module</t>
-        </is>
-      </c>
+          <t>CF_M01_AU33</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AU_33</t>
+          <t>AU_07</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CF_M01_AU29</t>
+          <t>CF_M01_AU10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D20" t="n">
         <v>1</v>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>API Gateway Service</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>The Web Socket service carries out the communication between the platform and the players.</t>
+          <t>This service is responsible for the management, authentication and authorization of platform users.</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2671,29 +2679,29 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>['AU_11', 'AU_27']</t>
+          <t>['AU_03', 'P_03']</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>AU_33</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>web socket, player</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr"/>
+          <t>AU_07</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>API Gateway Service</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>This service is responsible for communicating between the platform and the players.</t>
+          <t>This service is responsible for the management, authentication and authorization of platform users. It defines all the REST API routes and processes the requests to be sent to the Core service and the analytical module.</t>
         </is>
       </c>
       <c r="P20" t="n">
@@ -2701,112 +2709,108 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>CF_M01_AU27, CF_M01_AU14</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr">
         <is>
-          <t>CF_M01_AU29</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>player, web socket</t>
-        </is>
-      </c>
+          <t>CF_M01_AU10</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AU_34</t>
+          <t>AU_22</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CF_M01_AU28</t>
+          <t>CF_M01_AU17</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>connector</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D21" t="n">
         <v>1</v>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Amazon S3</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>The Api Player service communicates with the players receiving all the information corresponding to it.</t>
+          <t>This is the object storage service of AWS.</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>['AU_10', 'AU_27']</t>
+          <t>['AU_13']</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>AU_34</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>api player, player</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr"/>
+          <t>AU_22</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Amazon S3</t>
+        </is>
+      </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>This service is responsible for communicating with players.</t>
+          <t>This is the AWS object storage service. In this project it is responsible for storing JSON documents containing playlogs, connections and audit trails.</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>CF_M01_AU27, CF_M01_AU13</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr">
         <is>
-          <t>CF_M01_AU28</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>player, api player</t>
-        </is>
-      </c>
+          <t>CF_M01_AU17</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AU_20</t>
+          <t>AU_25</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CF_M01_AU33</t>
+          <t>CF_M01_AU21</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2819,7 +2823,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>NestJS</t>
+          <t>AWS Glue</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2829,29 +2833,29 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>As a framework, NestJS will be used.</t>
+          <t>The AWS Glue service is a serverless data integration service.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>49</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>['AU_03']</t>
+          <t>['AU_13']</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>AU_20</t>
+          <t>AU_25</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
-          <t>NestJS</t>
+          <t>AWS Glue</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2861,21 +2865,21 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>This framework is a NodeJS framework whose main function is to create backend applications. In this project, this framework has been used to develop the different services that interact with each other.</t>
+          <t>Serverless data integration service that allows us to detect, prepare, migrate and integrate data from different sources. In the case of the development of this project we have made use of the AWS Glue Data Catalog function. The use of this has been necessary to be able to store the metadata of the project data</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>CF_M01_AU02</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr">
         <is>
-          <t>CF_M01_AU33</t>
+          <t>CF_M01_AU21</t>
         </is>
       </c>
       <c r="T22" t="inlineStr"/>
@@ -2883,12 +2887,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AU_11</t>
+          <t>AU_03</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CF_M01_AU14</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2901,63 +2905,63 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Web Socket</t>
+          <t>Business Layer</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Layer</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>This service is responsible for carrying out the communication between the platform and the players, and in this way allows the exchange of information between them.</t>
+          <t>This layer is the core of the application and is responsible for processing all the information.</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>['AU_03']</t>
+          <t>['P_02']</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>AU_11</t>
+          <t>AU_03</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Web Socket</t>
+          <t>Business Layer</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Layer</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>This service is responsible for communicating between the platform and the players, thus allowing the exchange of information between them. It processes the data coming from the players and stores it in the database and in the cloud services.</t>
+          <t>This layer is the core of the application, which is responsible for processing all the information. In our context, it is the software that is responsible for processing user requests.</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_P02</t>
         </is>
       </c>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr">
         <is>
-          <t>CF_M01_AU14</t>
+          <t>CF_M01_AU06</t>
         </is>
       </c>
       <c r="T23" t="inlineStr"/>
@@ -2965,17 +2969,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AU_16</t>
+          <t>P_02</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CF_M01_AU17</t>
+          <t>CF_M01_P02</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>pattern</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -2983,63 +2987,63 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Amazon S3</t>
+          <t>Three Layers</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Architectural Pattern</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>This is the object storage service of AWS.</t>
+          <t>Pel model client-servidor s’utilitza l’arquitectura de 3 capes, on el sistema es devidiex en 3 capes, la capa de presentació, la capa de negoci i la capa de dades.</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>['AU_15']</t>
+          <t>['P_01']</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>AU_16</t>
+          <t>P_02</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Amazon S3</t>
+          <t>Three Layers</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Architectural Pattern</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>This is the AWS object storage service. In this project it is responsible for storing JSON documents containing playlogs, connections and audit trails.</t>
+          <t>The client-server model uses a 3-layer architecture, where the system is divided into 3 layers.</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_P01</t>
         </is>
       </c>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr">
         <is>
-          <t>CF_M01_AU17</t>
+          <t>CF_M01_P02</t>
         </is>
       </c>
       <c r="T24" t="inlineStr"/>
@@ -3047,12 +3051,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AU_24</t>
+          <t>AU_26</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CF_M01_AU21</t>
+          <t>CF_M01_AU22</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3065,7 +3069,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>AWS Glue</t>
+          <t>Kinesis Data Streams</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3075,29 +3079,29 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>The AWS Glue service is a serverless data integration service.</t>
+          <t>Kinesis Data Streams is a data processing and ingestion service aimed especially at data streaming.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>['AU_09']</t>
+          <t>['AU_13']</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>AU_24</t>
+          <t>AU_26</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
-          <t>AWS Glue</t>
+          <t>Kinesis Data Streams</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -3107,11 +3111,13 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Serverless data integration service that allows us to detect, prepare, migrate and integrate data from different sources. In the case of the development of this project we have made use of the AWS Glue Data Catalog function. The use of this has been necessary to be able to store the metadata of the project data</t>
-        </is>
-      </c>
-      <c r="P25" t="n">
-        <v>49</v>
+          <t>Data processing and ingestion service aimed especially at data streaming. In the development of this project, Kinesis Data Streams has been used to transmit playlog and audit trail data.</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>50, 51</t>
+        </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -3121,7 +3127,7 @@
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr">
         <is>
-          <t>CF_M01_AU21</t>
+          <t>CF_M01_AU22</t>
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
@@ -3129,17 +3135,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AU_03</t>
+          <t>P_01</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_P01</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>pattern</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -3147,17 +3153,17 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Business Layer</t>
+          <t>Client-Server</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Layer</t>
+          <t>Architectural Pattern</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>This layer is the core of the application and is responsible for processing all the information.</t>
+          <t>En el nostre projecte la plataforma de Waapiti és un servei web que segueix l’arquitectura client-servidor.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3165,45 +3171,37 @@
           <t>41</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>['P_02']</t>
-        </is>
-      </c>
+      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>AU_03</t>
+          <t>P_01</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Business Layer</t>
+          <t>Client-Server</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Layer</t>
+          <t>Architectural Pattern</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>This layer is the core of the application, which is responsible for processing all the information. In our context, it is the software that is responsible for processing user requests.</t>
+          <t>The Waapiti platform is a web service that follows the client-server architecture. In this type of architecture, the client is the one who makes requests to a server, which processes them and returns the response to the client.</t>
         </is>
       </c>
       <c r="P26" t="n">
         <v>41</v>
       </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>CF_M01_P02</t>
-        </is>
-      </c>
+      <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr">
         <is>
-          <t>CF_M01_AU06</t>
+          <t>CF_M01_P01</t>
         </is>
       </c>
       <c r="T26" t="inlineStr"/>
@@ -3211,17 +3209,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>P_02</t>
+          <t>AU_15</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CF_M01_P02</t>
+          <t>CF_M01_AU34</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>pattern</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -3229,63 +3227,63 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Three Layers</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Architectural Pattern</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Pel model client-servidor s’utilitza l’arquitectura de 3 capes, on el sistema es devidiex en 3 capes, la capa de presentació, la capa de negoci i la capa de dades.</t>
+          <t>With the language Typescript.</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>['P_01']</t>
+          <t>['AU_03']</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>P_02</t>
+          <t>AU_15</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Three Layers</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Architectural Pattern</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>The client-server model uses a 3-layer architecture, where the system is divided into 3 layers.</t>
+          <t>This programming language is built on top of JavaScript, it extends the JavaScript syntax.</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>CF_M01_P01</t>
+          <t>CF_M01_AU33</t>
         </is>
       </c>
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr">
         <is>
-          <t>CF_M01_P02</t>
+          <t>CF_M01_AU34</t>
         </is>
       </c>
       <c r="T27" t="inlineStr"/>
@@ -3293,12 +3291,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AU_25</t>
+          <t>AU_04</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CF_M01_AU22</t>
+          <t>CF_M01_AU07</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3311,65 +3309,63 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Kinesis Data Streams</t>
+          <t>Data Layer</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Layer</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Kinesis Data Streams is a data processing and ingestion service specifically aimed at data streaming.</t>
+          <t>It is the layer that is responsible for storing all the data.</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>['AU_08']</t>
+          <t>['P_02']</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>AU_25</t>
+          <t>AU_04</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Kinesis Data Streams</t>
+          <t>Data Layer</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Layer</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Data processing and ingestion service aimed especially at data streaming. In the development of this project, Kinesis Data Streams has been used to transmit playlog and audit trail data.</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>50, 51</t>
-        </is>
+          <t>It is the layer that is responsible for storing all the data. In our case, it would be the database and AWS storage services.</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>41</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>CF_M01_AU16</t>
+          <t>CF_M01_P02</t>
         </is>
       </c>
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr">
         <is>
-          <t>CF_M01_AU22</t>
+          <t>CF_M01_AU07</t>
         </is>
       </c>
       <c r="T28" t="inlineStr"/>
@@ -3377,17 +3373,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>P_01</t>
+          <t>AU_27</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CF_M01_P01</t>
+          <t>CF_M01_AU23</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>pattern</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -3395,55 +3391,63 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Client-Server</t>
+          <t>Kinesis Data Firehose</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Architectural Pattern</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>En el nostre projecte la plataforma de Waapiti és un servei web que segueix l’arquitectura client-servidor.</t>
+          <t>The Kinesis Data Firehose service has as its main function the loading of large amounts of data into data warehouses.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>41</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr"/>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>['AU_13']</t>
+        </is>
+      </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>P_01</t>
+          <t>AU_27</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Client-Server</t>
+          <t>Kinesis Data Firehose</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Architectural Pattern</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>The Waapiti platform is a web service that follows the client-server architecture. In this type of architecture, the client is the one who makes requests to a server, which processes them and returns the response to the client.</t>
+          <t>Its main function is to load large amounts of data into data warehouses. In this project we have used Kinesis Data Stream to store the playlogs and audit trail data in their corresponding S3 buckets. In addition, we have used one of the functionalities that Kinesis Data Firehose has with respect to the S3 service, which is dynamic partitioning.</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>41</v>
-      </c>
-      <c r="Q29" t="inlineStr"/>
+        <v>51</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>CF_M01_AU16</t>
+        </is>
+      </c>
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr">
         <is>
-          <t>CF_M01_P01</t>
+          <t>CF_M01_AU23</t>
         </is>
       </c>
       <c r="T29" t="inlineStr"/>
@@ -3451,12 +3455,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AU_21</t>
+          <t>AU_19</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CF_M01_AU34</t>
+          <t>CF_M01_AU31</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3469,7 +3473,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>TCP</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3479,29 +3483,29 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>With the language Typescript.</t>
+          <t>The communication between the API Gateway service is through the TCP communication protocol.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>['AU_20']</t>
+          <t>['AU_03', 'AU_31']</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>AU_21</t>
+          <t>AU_19</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>TCP</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3511,7 +3515,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>This programming language is built on top of JavaScript, it extends the JavaScript syntax.</t>
+          <t>communication between the Api Gateway service is via the TCP communication protocol</t>
         </is>
       </c>
       <c r="P30" t="n">
@@ -3519,262 +3523,16 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>CF_M01_AU33</t>
+          <t>CF_M01_AU26,CF_M01_AU27</t>
         </is>
       </c>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr">
         <is>
-          <t>CF_M01_AU34</t>
+          <t>CF_M01_AU31</t>
         </is>
       </c>
       <c r="T30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>AU_04</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>CF_M01_AU07</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Data Layer</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Layer</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>It is the layer that is responsible for storing all the data.</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>41</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>['P_02']</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>AU_04</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>Data Layer</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>Layer</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>It is the layer that is responsible for storing all the data. In our case, it would be the database and AWS storage services.</t>
-        </is>
-      </c>
-      <c r="P31" t="n">
-        <v>41</v>
-      </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>CF_M01_P02</t>
-        </is>
-      </c>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>CF_M01_AU07</t>
-        </is>
-      </c>
-      <c r="T31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>AU_26</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>CF_M01_AU23</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Kinesis Data Firehose</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>The Kinesis Data Firehose service has as its main function the loading of large amounts of data into data warehouses.</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>51</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>['AU_08']</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>AU_26</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>Kinesis Data Firehose</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>Its main function is to load large amounts of data into data warehouses. In this project we have used Kinesis Data Stream to store the playlogs and audit trail data in their corresponding S3 buckets. In addition, we have used one of the functionalities that Kinesis Data Firehose has with respect to the S3 service, which is dynamic partitioning.</t>
-        </is>
-      </c>
-      <c r="P32" t="n">
-        <v>51</v>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>CF_M01_AU16</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>CF_M01_AU23</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>AU_19</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>CF_M01_AU31</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>TCP</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>The communication between the API Gateway service is through the TCP communication protocol.</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>['AU_07']</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>AU_19</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>TCP</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>communication between the Api Gateway service is via the TCP communication protocol</t>
-        </is>
-      </c>
-      <c r="P33" t="n">
-        <v>44</v>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>CF_M01_AU26,CF_M01_AU27</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>CF_M01_AU31</t>
-        </is>
-      </c>
-      <c r="T33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3787,7 +3545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3871,147 +3629,151 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AU_15</t>
+          <t>AU_16</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Data Lake</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>The objective of these services is to form a data lake where all the history is stored to be able to process them in the analytical module.</t>
+          <t>For the infrastructure, the cloud services of AWS will be used.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>CF_M01_AU07</t>
+          <t>CF_M01_AU16</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Data Layer</t>
+          <t>AWS cloud services set</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.7526</v>
+        <v>0.8603</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AU_30</t>
+          <t>AU_21</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Connector</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>core, relational database</t>
-        </is>
-      </c>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Amazon RDS</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>The Core service interacts with the database, although it also interacts to a lesser extent with cloud services.</t>
+          <t>This database is implemented in the RDS service.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>CF_M01_AU11</t>
+          <t>CF_M01_AU18</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Core Service</t>
+          <t>Amazon DynamoDB</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0.7699</v>
+        <v>0.7803</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AU_31</t>
+          <t>AU_28</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Connector</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>analytical module, data lake</t>
-        </is>
-      </c>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>AWS CDK</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>The analytical module interacts with cloud services, although it also interacts to a lesser extent with the database.</t>
+          <t>The AWS CDK is the AWS framework that allows the construction of applications in the cloud.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>CF_M01_AU12</t>
+          <t>CF_M01_AU18</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Analytical module</t>
+          <t>Amazon DynamoDB</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.7214</v>
+        <v>0.7153</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AU_32</t>
+          <t>AU_29</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Connector</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>web socket, relational database, data lake</t>
-        </is>
-      </c>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>AWS CloudFormation</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>The Web Socket service processes data from players and stores it in the database and cloud services.</t>
+          <t>AWS CloudFormation is an Amazon service that helps configure AWS resources.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>CF_M01_AU29</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>CF_M01_AU16</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>AWS cloud services set</t>
+        </is>
+      </c>
       <c r="H6" t="n">
-        <v>0.799</v>
+        <v>0.7708</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AU_35</t>
+          <t>AU_32</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4022,32 +3784,28 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>analytical module, amazon athena, amazon s3</t>
+          <t>web socket service, player api service</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>The analytical module uses Amazon Athena to perform queries on data stored in Amazon S3.</t>
+          <t>Aquest servei [Web Socket] s’encarrega de realitzar la comunicació entre la plataforma i els players, i d’aquesta manera permet l’intercanvi d’informació entre ells.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CF_M01_AU17</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Amazon S3</t>
-        </is>
-      </c>
+          <t>CF_M01_AU29</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>0.7788</v>
+        <v>0.847</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AU_36</t>
+          <t>AU_33</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4058,98 +3816,58 @@
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>core, web socket, kinesis data streams</t>
+          <t>web socket service, database, aws cloud services</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>The microservices (Core and Web Socket) send data to the Kinesis Data Stream.</t>
+          <t>Processa les dades provinents dels players i les emmagatzema en la base de dades i en els serveis cloud.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>CF_M01_AU22</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Kinesis Data Streams</t>
-        </is>
-      </c>
+          <t>CF_M01_AU29</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>0.7889</v>
+        <v>0.7296</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AU_37</t>
+          <t>P_04</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Connector</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>kinesis data firehose, kinesis data streams, amazon s3</t>
-        </is>
-      </c>
+          <t>Design Pattern</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Microservices</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Kinesis Data Firehose reads from the Kinesis Data Stream and saves the data in Amazon S3.</t>
+          <t>En el cas de la plataforma de Waapiti, l’arquitectura física no es correspon exactament a l’arquitectura lògica, ja que tant la capa de negoci com la capa de dades es divideixen en diversos serveis diferents.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>CF_M01_AU23</t>
+          <t>CF_M01_AU10</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Kinesis Data Firehose</t>
+          <t>API Gateway Service</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0.8948</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>P_04</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Design Pattern</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Data lake</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Un data lake consisteix en un dipòsit de dades que poden ser emmagatzemades en el seu format natural.</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>CF_M01_AU07</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Data Layer</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>0.7534</v>
+        <v>0.7454</v>
       </c>
     </row>
   </sheetData>
@@ -4163,7 +3881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4211,43 +3929,43 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CF_M01_AU01</t>
+          <t>CF_M01_AU27</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>Player</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>The client is the user of the platform</t>
+          <t>A player consists of a device that can be internal or external, which allows screens to reproduce content on the screens.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>P_01</t>
+          <t>AU_01</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Client-Server</t>
+          <t>User</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0.8333</v>
+        <v>0.7565</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CF_M01_AU02</t>
+          <t>CF_M01_AU01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4257,13 +3975,13 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Server</t>
+          <t>Client</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>The server is the software that is responsible for processing user requests.</t>
+          <t>The client is the user of the platform</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -4277,62 +3995,62 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.8237</v>
+        <v>0.8333</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CF_M01_AU24</t>
+          <t>CF_M01_AU02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Connector</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Internet</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>client, server</t>
-        </is>
-      </c>
+          <t>Server</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Communication between the two components is carried out over the internet using the HTTP protocol and the REST API model.</t>
+          <t>The server is the software that is responsible for processing user requests.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>AU_28</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>P_01</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Client-Server</t>
+        </is>
+      </c>
       <c r="H4" t="n">
-        <v>0.8183</v>
+        <v>0.8237</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CF_M01_AU04</t>
+          <t>CF_M01_AU24</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>REST</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>client, server</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>Communication between the two components is carried out over the internet using the HTTP protocol and the REST API model.</t>
@@ -4340,7 +4058,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>AU_18</t>
+          <t>AU_17</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -4349,7 +4067,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.6758999999999999</v>
+        <v>0.7941</v>
       </c>
     </row>
     <row r="6">
@@ -4391,37 +4109,137 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>CF_M01_AU28</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>player, api player</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>This service is responsible for communicating with players.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>AU_32</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>0.8078</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CF_M01_AU29</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>player, web socket</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>This service is responsible for communicating between the platform and the players.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>AU_32</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>0.847</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CF_M01_AU35</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>AWSS RDS</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>This database is implemented in the RDS service [30], which is a distributed relational database service from AWS.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>AU_21</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Amazon RDS</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>0.742</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>CF_M01_P03</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Architectural Pattern</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Service-oriented</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
         <is>
           <t>Both the business layer and the data layer are divided into several different services</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>P_01</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Client-Server</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>0.703</v>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>AU_08</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Core Service</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>0.766</v>
       </c>
     </row>
   </sheetData>

</xml_diff>